<commit_message>
Replace non-question focus keys with question keys in content plans
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -1038,12 +1038,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Продаж кредитної квартири: як це робиться</t>
+          <t>Чи можна купити квартиру, якщо у продавця є борги по кредитах</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>продажа кредитной квартиры</t>
+          <t>можно ли купить квартиру если есть долги по кредитам</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1096,12 +1096,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Суд по іпотеці: як відбувається і що робити боржнику</t>
+          <t>Як взяти відстрочку по іпотеці: що подати в банк</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>суд по ипотеке</t>
+          <t>как взять отсрочку по ипотеке</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Перекредитування під заставу нерухомості: коли вигідно</t>
+          <t>Як взяти іпотеку з поганою кредитною історією</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>перекредитование под залог недвижимости</t>
+          <t>плохая кредитная история как взять ипотеку</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Кредитні канікули від держави: хто може скористатися</t>
+          <t>Як оформити кредитні канікули в МФО</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>кредитные каникулы от государства</t>
+          <t>как оформить кредитные каникулы в мфо</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Чи можна платити мікрозайм частинами</t>
+          <t>Як закрити мікрозайм, якщо немає грошей</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>можно ли платить микрозайм частями</t>
+          <t>как закрыть микрозайм если нет денег</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Як закрити мікрозайм, якщо немає грошей</t>
+          <t>Чи можна платити мікрозайм частинами</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>как закрыть микрозайм если нет денег</t>
+          <t>можно ли платить микрозайм частями</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2291,12 +2291,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Клопотання про застосування строку позовної давності по кредиту</t>
+          <t>Що таке строк позовної давності за кредитом і як його застосувати в суді</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>ходатайство о применении срока исковой давности по кредиту</t>
+          <t>что такое срок исковой давности по кредиту</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -2320,12 +2320,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Суд із ПриватБанком по кредитній картці: як розірвати договір</t>
+          <t>Як боротися з ПриватБанком у суді по кредитній картці</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>суд с приватбанком и как разорвать договор по кредитке</t>
+          <t>как бороться с приватбанком</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2407,12 +2407,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Кейс: наслідки суду по кредиту для боржника</t>
+          <t>Чим загрожує суд по кредиту: наслідки для боржника</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>последствия суда по кредиту</t>
+          <t>чем грозит суд по кредиту</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2960,12 +2960,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Рішення суду про стягнення заборгованості за кредитним договором: що в ньому перевірити</t>
+          <t>Хто судився з ПриватБанком по кредитній картці: практика та результати</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>решение суда о взыскании задолженности по кредитному договору</t>
+          <t>кто судился с приватбанком</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3078,12 +3078,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Прострочки в МФО: що робити</t>
+          <t>Як поводитися з МФО при простроченні</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>просрочки в мфо что делать</t>
+          <t>как вести себя с мфо при просрочке</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -3747,12 +3747,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Розірвання кредитного договору через суд</t>
+          <t>Чи можна розірвати кредитний договір з банком</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>расторжение кредитного договора через суд</t>
+          <t>можно ли расторгнуть кредитный договор с банком</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4155,12 +4155,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Заява на закриття кредиту: як написати</t>
+          <t>Які документи потрібні для закриття кредиту</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>заявление на закрытие кредита</t>
+          <t>какие документы нужны для закрытия кредита</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4273,12 +4273,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо не платити кредит: наслідки прострочення</t>
+          <t>Що буде за прострочку кредиту: наслідки для позичальника</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>просрочка по кредиту последствия</t>
+          <t>что будет за просрочку кредита</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4331,12 +4331,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Як оскаржити кредитний договір: підстави та судова практика</t>
+          <t>Як оскаржити кредитний договір з банком: підстави та судова практика</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>оспаривание кредитного договора</t>
+          <t>как оспорить кредитный договор с банком</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4505,12 +4505,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: реструктуризація боргу в МФО — як домовитися про графік платежів</t>
+          <t>Кейс: як реструктуризувати мікрозайм і домовитися про графік платежів</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>реструктуризация долга в мфо</t>
+          <t>как реструктуризировать микрозаймы</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -6342,12 +6342,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Банкрутство при боргах у МФО: чи можливе</t>
+          <t>Що буде, якщо оголосити себе банкрутом: наслідки для фізособи</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>банкротство мфо</t>
+          <t>что если объявить себя банкротом</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -6371,12 +6371,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Стягнення заборгованості з банкрута</t>
+          <t>Що потрібно, щоб оголосити себе банкрутом: умови та документи</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>взыскание задолженности с банкрота</t>
+          <t>что надо чтобы объявить себя банкротом</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove case-type articles from content plans
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як дізнатися, чи знято арешт з квартири</t>
+          <t>Як дізнатися, чи знято арешт з квартири</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як перевірити, чи накладено арешт на квартиру</t>
+          <t>Як перевірити, чи накладено арешт на квартиру</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як повернути кредитний автомобіль банку</t>
+          <t>Як повернути кредитний автомобіль банку</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як знизити ставку за кредитом</t>
+          <t>Як знизити ставку за кредитом</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як сплатити лише тіло кредиту в МФО</t>
+          <t>Як сплатити лише тіло кредиту в МФО</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: що означає «заморозити» позику</t>
+          <t>Що означає «заморозити» позику</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: на які рахунки не можна накладати арешт</t>
+          <t>На які рахунки не можна накладати арешт</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як дізнатися, арештовано рахунок чи ні</t>
+          <t>Як дізнатися, арештовано рахунок чи ні</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: через скільки знімається арешт із картки після оплати</t>
+          <t>Через скільки знімається арешт із картки після оплати</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи можна виграти суд у банку</t>
+          <t>Чи можна виграти суд у банку</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи може суд скасувати відсотки по кредиту</t>
+          <t>Чи може суд скасувати відсотки по кредиту</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як подати позов до суду на МФО</t>
+          <t>Як подати позов до суду на МФО</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: через який час МФО подає до суду</t>
+          <t>Через який час МФО подає до суду</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи нараховуються відсотки після рішення суду</t>
+          <t>Чи нараховуються відсотки після рішення суду</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: борги у кількох банках — як діяти</t>
+          <t>Борги у кількох банках — як діяти</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Кейс: великий борг у мікрозаймі — що робити</t>
+          <t>Великий борг у мікрозаймі — що робити</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи можуть відсотки перевищувати суму позики</t>
+          <t>Чи можуть відсотки перевищувати суму позики</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як нараховуються відсотки по кредитній картці</t>
+          <t>Як нараховуються відсотки по кредитній картці</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як правильно закрити кредитну картку</t>
+          <t>Як правильно закрити кредитну картку</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: у банку немає оригіналу кредитного договору</t>
+          <t>У банку немає оригіналу кредитного договору</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як погасити кредит, якщо картку заблоковано</t>
+          <t>Як погасити кредит, якщо картку заблоковано</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -4097,7 +4097,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: що буде, якщо не платити кредит за телефон</t>
+          <t>Що буде, якщо не платити кредит за телефон</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як отримати довідку про закриття кредиту</t>
+          <t>Як отримати довідку про закриття кредиту</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -4418,7 +4418,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як зменшити суму платежу за кредитом через переговори з банком</t>
+          <t>Як зменшити суму платежу за кредитом через переговори з банком</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як реструктуризувати мікрозайм і домовитися про графік платежів</t>
+          <t>Як реструктуризувати мікрозайм і домовитися про графік платежів</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: що буде, якщо не платити кредит під заставу нерухомості</t>
+          <t>Що буде, якщо не платити кредит під заставу нерухомості</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як скасувати виконавче провадження за кредитом</t>
+          <t>Як скасувати виконавче провадження за кредитом</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як діяти боржнику, якщо є рішення суду про стягнення</t>
+          <t>Як діяти боржнику, якщо є рішення суду про стягнення</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: рішення суду по кредиту — що робити далі</t>
+          <t>Рішення суду по кредиту — що робити далі</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи дадуть кредит, якщо є прострочка по іншому кредиту</t>
+          <t>Чи дадуть кредит, якщо є прострочка по іншому кредиту</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи може банк вимагати повернути весь кредит одразу</t>
+          <t>Чи може банк вимагати повернути весь кредит одразу</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -5408,7 +5408,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як оскаржити комісію банку</t>
+          <t>Як оскаржити комісію банку</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -5613,7 +5613,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи можуть колектори заборонити виїзд за кордон</t>
+          <t>Чи можуть колектори заборонити виїзд за кордон</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи можуть забрати пенсію за кредит</t>
+          <t>Чи можуть забрати пенсію за кредит</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: що робити з кредитом, якщо людина у в’язниці</t>
+          <t>Що робити з кредитом, якщо людина у в’язниці</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -6050,7 +6050,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи варто ховатися від кредиторів</t>
+          <t>Чи варто ховатися від кредиторів</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -6137,7 +6137,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: втратив роботу — як платити кредит</t>
+          <t>Втратив роботу — як платити кредит</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи може банк «забути» про кредит</t>
+          <t>Чи може банк «забути» про кредит</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -6516,7 +6516,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як зупинити дзвінки колекторів</t>
+          <t>Як зупинити дзвінки колекторів</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -6526,7 +6526,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Кейс: дзвінки колекторів за чужим кредитом — як позбутися</t>
+          <t>Дзвінки колекторів за чужим кредитом — як позбутися</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як розмовляти з колекторами, якщо немає грошей</t>
+          <t>Як розмовляти з колекторами, якщо немає грошей</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: чи спишуть борги по кредитах пенсіонерам</t>
+          <t>Чи спишуть борги по кредитах пенсіонерам</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як позбутися кредитних боргів законно</t>
+          <t>Як позбутися кредитних боргів законно</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -7040,7 +7040,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: куди звернутися, щоб списали кредит</t>
+          <t>Куди звернутися, щоб списали кредит</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -7274,7 +7274,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Кейс: як довести, що ти не брав кредит</t>
+          <t>Як довести, що ти не брав кредит</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -7390,7 +7390,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Кейс: куди звертатися, якщо на мене оформили кредит</t>
+          <t>Куди звертатися, якщо на мене оформили кредит</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -7400,7 +7400,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -7448,7 +7448,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Кейс: що робити, якщо втратили кредитний договір</t>
+          <t>Що робити, якщо втратили кредитний договір</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Кейс</t>
+          <t>Розбір питання</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Content plans: focus phrase is the semantic key, add frequency and cluster columns
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -71,12 +71,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -952,9 +955,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -976,17 +979,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1009,17 +1012,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Чим небезпечний кредит під заставу квартири</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>чем опасен кредит под залог квартиры</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>828000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>чем опасен кредит под залог квартиры</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1038,17 +1039,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Чи можна купити квартиру, якщо у продавця є борги по кредитах</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>можно ли купить квартиру если есть долги по кредитам</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>121000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли купить квартиру если есть долги по кредитам</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -1067,17 +1066,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Чи можна продати квартиру, якщо є борги по кредитах</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>можно ли продать квартиру если есть долги по кредитам</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>17700000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли продать квартиру если есть долги по кредитам</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1096,17 +1093,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як взяти відстрочку по іпотеці: що подати в банк</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как взять отсрочку по ипотеке</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>66</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что значит заморозить займ</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -1125,17 +1120,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як взяти іпотеку з поганою кредитною історією</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>плохая кредитная история как взять ипотеку</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>5430000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1154,17 +1147,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, чи знято арешт з квартири</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>как узнать снят ли арест с квартиры</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>5730000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как проверить арест на движимое имущество</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -1183,17 +1174,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Як зняти арешт з автомобіля, накладений судом</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>как снять арест с автомобиля наложенный судом</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>9740</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как вернуть кредитную машину</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1212,17 +1201,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Чи можна продати авто, яке в кредиті</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>можно ли продать авто которое в кредите</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>198</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли обменять кредитную машину на другую</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -1241,17 +1228,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як перевірити, чи накладено арешт на квартиру</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как проверить наложен ли арест на квартиру</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>14100000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как проверить арест на движимое имущество</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1270,17 +1255,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Як зняти заставу з авто після погашення кредиту</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>как снять залог с авто после погашения кредита</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>99</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как вернуть кредитную машину</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -1299,17 +1282,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо на машину накладено арешт</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>что делать если на машину наложен арест</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>133000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как вернуть кредитную машину</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1328,17 +1309,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Як повернути кредитний автомобіль банку</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>как вернуть кредитный автомобиль банку</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>7710000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как вернуть кредитный автомобиль банку</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1360,9 +1339,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1384,17 +1363,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1417,17 +1396,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як попросити в банку відстрочку за кредитом</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как попросить у банка отсрочку по кредиту</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>354000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что значит заморозить займ</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1446,17 +1423,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Як отримати кредитні канікули в банку</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>как получить кредитные каникулы в банке</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>93</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что значит заморозить займ</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -1475,17 +1450,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Як оформити кредитні канікули в МФО</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>как оформить кредитные каникулы в мфо</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>415000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что значит заморозить займ</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1504,17 +1477,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як написати лист у банк про відстрочку платежу</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как написать письмо в банк об отсрочке платежа</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>1640000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что значит заморозить займ</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -1533,17 +1504,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як знизити ставку за кредитом</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как снизить ставку по кредиту</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>6710000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как снизить ставку по кредиту</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1562,17 +1531,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Як домовитися з МФО про розстрочку</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>как договориться с мфо о рассрочке</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>632000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -1591,17 +1558,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Як домовитися з МФО про списання відсотків</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>как договориться с мфо о списании процентов</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>49000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>помощь в закрытии долгов</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1620,17 +1585,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Як сплатити лише тіло кредиту в МФО</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>100</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -1649,17 +1612,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як закрити мікрозайм, якщо немає грошей</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как закрыть микрозайм если нет денег</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>111</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1678,17 +1639,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи можна платити мікрозайм частинами</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>можно ли платить микрозайм частями</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>40800</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -1707,17 +1666,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Як краще закрити кредит достроково</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>как лучше закрыть кредит досрочно</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>656000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как лучше закрыть кредит досрочно</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1736,17 +1693,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Що означає «заморозити» позику</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>что значит заморозить займ</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>56600</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что значит заморозить займ</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1768,9 +1723,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1792,17 +1747,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1825,17 +1780,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, чи є ви в реєстрі боржників</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как узнать есть ли ты в реестре должников</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>300</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как убрать себя с реестра должников</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -1854,17 +1807,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Як прибрати себе з реєстру боржників</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>как убрать себя с реестра должников</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>226000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как убрать себя с реестра должников</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -1883,17 +1834,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо висить борг у державних виконавців</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>если висит долг у судебных приставов</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>105</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>если висит долг у судебных приставов</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -1912,17 +1861,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть пристави заарештувати рахунок без суду</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>могут ли арестовать счета без суда</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>441000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -1941,17 +1888,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Які виплати не підлягають арешту</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>какие выплаты не подлежат аресту</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>1680000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1970,17 +1915,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>На які рахунки не можна накладати арешт</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>на какие счета нельзя накладывать арест</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>321000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -1999,17 +1942,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Чи можна користуватися карткою, якщо на ній арешт</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>можно ли пользоваться картой если на ней арест</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>50800</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -2028,17 +1969,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Як отримувати зарплату, якщо картку арештовано</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>как получать зарплату если карта арестована</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>200</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -2057,17 +1996,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як зняти арешт із зарплатної картки</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>можно ли снять арест с зарплатной карты</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>63800</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -2086,17 +2023,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, арештовано рахунок чи ні</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>как узнать арестован счет или нет</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>4520000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как проверить арест на движимое имущество</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -2115,17 +2050,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Чи можна арештувати дитячу допомогу</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>имеют ли право наложить арест на детское пособие</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>130000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -2144,17 +2077,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Через скільки знімається арешт із картки після оплати</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>через сколько снимается арест с карты после оплаты</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>326000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -2176,9 +2107,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2200,17 +2131,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -2233,17 +2164,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як скасувати рішення суду по кредиту</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как отменить решение суда по кредиту</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>3590000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как отменить решение суда по кредиту</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -2262,17 +2191,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Апеляція на рішення суду по кредиту: строки і порядок</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>апелляция на решение суда по кредиту</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>73</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>апелляция на решение суда по кредиту</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -2291,17 +2218,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Що таке строк позовної давності за кредитом і як його застосувати в суді</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>что такое срок исковой давности по кредиту</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>300</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>срок исковой давности по кредиту в приватбанке</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -2320,17 +2245,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як боротися з ПриватБанком у суді по кредитній картці</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как бороться с приватбанком</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>1160000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд с приватбанком и как разорвать договор по кредитке</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -2349,17 +2272,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, хто подав до суду по кредиту</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как узнать кто подал в суд по кредиту</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>93</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как узнать кто подал в суд по кредиту</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -2378,17 +2299,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Повістка до суду за несплату кредиту: що робити</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>повестка в суд за неуплату кредита</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>122000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>повестка в суд за неуплату кредита</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -2407,17 +2326,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Чим загрожує суд по кредиту: наслідки для боржника</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>чем грозит суд по кредиту</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>84700</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>просрочка по кредиту последствия</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -2436,17 +2353,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Чому банк не подає до суду по кредиту</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>почему банк не подает в суд по кредиту</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>14400000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>почему банк не подает в суд по кредиту</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -2465,17 +2380,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Що говорити в суді по кредиту</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>что говорить в суде по кредиту</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>492000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд по ипотеке</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -2494,17 +2407,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи можна виграти суд у банку</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>можно ли выиграть суд с банком</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>3280000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд по ипотеке</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -2523,17 +2434,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Як оскаржити відсотки по кредиту в суді</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>как оспорить проценты по кредиту в суде</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>5010000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -2552,17 +2461,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Чи може суд скасувати відсотки по кредиту</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>может ли суд отменить проценты по кредиту</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>693000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -2584,9 +2491,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2608,17 +2515,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -2641,17 +2548,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Банк звернувся до суду: що робити боржнику</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>банк обратился в суд что делать</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>27500000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд по ипотеке</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -2670,17 +2575,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Як поводитися в суді з банком</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>как вести себя в суде с банком</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд по ипотеке</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -2699,17 +2602,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Як оскаржити рішення суду по мікрозаймах</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>как оспорить решение суда по микрозаймам</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>1600000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -2728,17 +2629,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як виграти суд у мікрофінансової організації</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как выиграть суд у микрофинансовой организации</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>66100</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -2757,17 +2656,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як подати позов до суду на МФО</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>1810000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -2786,17 +2683,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Чи можна подати до суду на банк</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>можно ли подать в суд на банк</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>21800000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд по ипотеке</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -2815,17 +2710,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Як судитися з МФО: покрокова інструкція</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>как судиться с мфо</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>11100000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -2844,17 +2737,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Якщо МФО подало до суду: що робити</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>если мфо подала в суд</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>51600</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>які мікрозайми подають в суд</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -2873,17 +2764,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Через який час МФО подає до суду</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>через какое время мфо подает в суд</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>270000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -2902,17 +2791,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Як знизити відсотки по мікрозайму через суд</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>как снизить проценты по микрозайму в суде</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>54400</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -2931,17 +2818,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Чи нараховуються відсотки після рішення суду</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>начисляются ли проценты по кредиту после решения суда</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>2510000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -2960,17 +2845,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Хто судився з ПриватБанком по кредитній картці: практика та результати</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>кто судился с приватбанком</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>859000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд с приватбанком и как разорвать договор по кредитке</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -2992,9 +2875,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3016,17 +2899,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3049,17 +2932,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо не можеш виплатити позику</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>что делать если не можешь выплатить займ</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>122</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -3078,17 +2959,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Як поводитися з МФО при простроченні</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>как вести себя с мфо при просрочке</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>3020000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>чего боятся мфо украины</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -3107,17 +2986,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Куча боргів у МФО: з чого почати</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>куча долгов в мфо что делать</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>50600</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -3136,17 +3013,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо взято багато позик</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>что делать если много займов</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>612000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как подать иск в суд на мфо</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -3165,17 +3040,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Борги у кількох банках — як діяти</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>если долги в нескольких банках</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какие кредиты списывают</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -3194,17 +3067,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Хто може допомогти з боргами</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>кто может помочь с долгами</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>48000000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какие кредиты списывают</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -3223,17 +3094,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Що таке мікрокредитування і чим воно небезпечне</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>что такое микрокредитование и чем оно опасно</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>85</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что такое микрокредитование и чем оно опасно</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -3252,17 +3121,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Великий борг у мікрозаймі — що робити</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>большой долг в микрозайме что делать</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>86500</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -3281,17 +3148,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Скільки максимум відсотків можуть нарахувати МФО</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>сколько максимум процентов может начислить мфо</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>34900</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -3310,17 +3175,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи може пеня перевищувати суму боргу</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>может ли пеня превышать сумму долга</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>1150000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -3339,17 +3202,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть відсотки перевищувати суму позики</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>могут ли проценты превышать сумму займа</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>286000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -3368,17 +3229,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Як порахувати відсоток прострочки по кредиту</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>как посчитать процент просрочки по кредиту</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>587000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>просрочка по кредиту последствия</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -3400,9 +3259,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3424,17 +3283,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3457,17 +3316,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як зробити реструктуризацію кредиту в ПриватБанку</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как сделать реструктуризацию кредита в приватбанке</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>2270</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -3486,17 +3343,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Борг у ПриватБанку: що робити</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>долг в приватбанке что делать</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>153000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>кредитка приватбанка штраф</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -3515,17 +3370,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, чи є борг у ПриватБанку</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>как узнать есть ли долг в приватбанке</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>502000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>кредитка приватбанка штраф</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -3544,17 +3397,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як погасити кредит у ПриватБанку, якщо немає грошей</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как погасить кредит в приватбанке если нет денег</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>194000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>кредитка приватбанка штраф</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -3573,17 +3424,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як нараховуються відсотки по кредитній картці</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как начисляются проценты по кредитной карте приватбанка</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>62</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>кредитка приватбанка штраф</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -3602,17 +3451,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо не сплачувати кредитну картку</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>что будет если не оплачивать кредитную карту</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>194000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>кредитка приватбанка штраф</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -3631,17 +3478,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Чи може банк списати борг</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>может ли приват банк списать долг</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>192000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -3660,17 +3505,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Як розрахувати обов’язковий платіж по кредитній картці</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>как рассчитать обязательный платеж по кредитной карте приватбанка</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>66</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>кредитка приватбанка штраф</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -3689,17 +3532,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як правильно закрити кредитну картку</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как правильно закрыть кредитку приватбанка</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>117000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>срок исковой давности по кредиту в приватбанке</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -3718,17 +3559,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Що таке пролонгація кредиту</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>что значит пролонгация кредита</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>240000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>пролонгация микрозайма</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -3747,17 +3586,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Чи можна розірвати кредитний договір з банком</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>можно ли расторгнуть кредитный договор с банком</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>314000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>оспаривание кредитного договора</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -3776,17 +3613,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>У банку немає оригіналу кредитного договору</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>если у банка нет оригинала кредитного договора</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>4290000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>оспаривание кредитного договора</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -3808,9 +3643,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3832,17 +3667,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3865,17 +3700,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Переплатила по кредиту: що робити</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>переплатила кредит что делать</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>3270000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>переплатила кредит что делать</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -3894,17 +3727,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Як повернути частину грошей за кредит</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>как вернуть часть денег за кредит</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>12500000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как вернуть часть денег за кредит</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -3923,17 +3754,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Чи потрібно йти в банк після погашення кредиту</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>нужно ли идти в банк после погашения кредита</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>3030000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>нужно ли идти в банк после погашения кредита</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -3952,17 +3781,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Чи потрібно писати заяву про дострокове погашення кредиту</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>нужно ли писать заявление на досрочное погашение кредита</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>1920000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>нужно ли писать заявление на досрочное погашение кредита</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -3981,17 +3808,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як погасити кредит, якщо картку заблоковано</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как погасить кредит если карта заблокирована</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>65000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как погасить кредит если карта заблокирована</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -4010,17 +3835,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Чи можна погасити кредит і одразу взяти новий</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>можно ли погасить кредит и сразу взять новый</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>2830000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли погасить кредит и сразу взять новый</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -4039,17 +3862,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо закінчився строк дії кредитної картки</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>что делать если срок действия кредитной карты истек</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>387000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что делать если срок действия кредитной карты истек</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -4068,17 +3889,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Чи можна погасити кредит через місяць</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>можно ли погасить кредит через месяц</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>4520000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли погасить кредит и сразу взять новый</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -4097,17 +3916,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо не платити кредит за телефон</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>что будет если не платить кредит за телефон</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>28900000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что будет если не платить кредит за телефон</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -4126,17 +3943,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи може банк списати борг із зарплатної картки</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>может ли банк списать долг по кредиту с зарплатной карты</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>11200000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -4155,17 +3970,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Які документи потрібні для закриття кредиту</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>какие документы нужны для закрытия кредита</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>6140000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>заявление на закрытие кредита</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -4184,17 +3997,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Як отримати довідку про закриття кредиту</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>как взять справку о закрытии кредита</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>79800</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>заявление на закрытие кредита</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -4216,9 +4027,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4240,17 +4051,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -4273,17 +4084,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Що буде за прострочку кредиту: наслідки для позичальника</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>что будет за просрочку кредита</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>5770000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>просрочка по кредиту последствия</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -4302,17 +4111,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть посадити за несплату кредиту в Україні</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>могут ли за долги посадить</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>310000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли за долги посадить</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -4331,17 +4138,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Як оскаржити кредитний договір з банком: підстави та судова практика</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>как оспорить кредитный договор с банком</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>478000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>оспаривание кредитного договора</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -4360,17 +4165,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Банк передав справу колекторам: що робити позичальнику</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>банк передал дело коллекторам что делать</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>1000000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>банк передал дело коллекторам что делать</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -4389,17 +4192,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть пристави заблокувати кредитну картку</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>могут ли заблокировать кредитную карту приставы</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>323000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли заблокировать кредитную карту приставы</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -4418,17 +4219,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Як зменшити суму платежу за кредитом через переговори з банком</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>как уменьшить сумму платежа по кредиту</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>200</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить сумму платежа по кредиту</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -4447,17 +4246,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Чи можна не платити кредит, якщо минуло 3 роки (позовна давність)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>можно ли не платить кредит если прошло 3 года</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>9670000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли не платить кредит если прошло 3 года</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -4476,17 +4273,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Прийшов судовий наказ про стягнення заборгованості за кредитом: що робити</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>пришел судебный приказ о взыскании задолженности по кредиту</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>279000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>пришел судебный приказ о взыскании задолженности по кредиту</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -4505,17 +4300,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як реструктуризувати мікрозайм і домовитися про графік платежів</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как реструктуризировать микрозаймы</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>340000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>реструктуризация займа в микрофинансовой организации</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -4534,17 +4327,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть колектори накласти арешт на майно</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>могут ли коллекторы наложить арест на имущество</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>235000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли коллекторы наложить арест на имущество</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -4563,17 +4354,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Якщо чоловік не платить кредит: що загрожує дружині</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>если муж не платит кредит что грозит жене</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>630000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>если муж не платит кредит что грозит жене</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -4592,17 +4381,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо не платити кредит під заставу нерухомості</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>что будет если не платить кредит под залог недвижимости</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>7180000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что будет если не платить кредит под залог недвижимости</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -4624,9 +4411,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4648,17 +4435,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -4681,17 +4468,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо не платити за виконавчим листом</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>что будет если не платить по исполнительному листу</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>4010000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -4710,17 +4495,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Чи можна домовитися з приставами про розстрочку боргу</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>можно ли договориться с приставами</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>695000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -4739,17 +4522,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Прийшов виконавчий лист за кредитом: що робити далі</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>что делать если пришел исполнительный лист по кредиту</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>198</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -4768,17 +4549,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як зменшити суму відрахувань за виконавчим листом</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>27800</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -4797,17 +4576,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як скасувати виконавче провадження за кредитом</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как отменить исполнительное производство по кредиту</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>13400000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -4826,17 +4603,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Як припинити виконавче провадження, якщо борг уже погашено</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>как прекратить исполнительное производство если долг погашен</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>26500</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -4855,17 +4630,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Чи можна скасувати виконавчий лист</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>можно ли отменить исполнительный лист</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>232000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -4884,17 +4657,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Як закрити заборгованість у державних виконавців</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>как закрыть задолженность у судебных приставов</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>614000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -4913,17 +4684,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як діяти боржнику, якщо є рішення суду про стягнення</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как не платить долг по решению суда</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>9580000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -4942,17 +4711,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть пристави списати всі гроші із зарплатної картки</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>могут ли приставы снимать все деньги с зарплатной карты</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>23500</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -4971,17 +4738,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Що робити з виконавчим листом: покрокова інструкція для боржника</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>что делать с исполнительным листом</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>10800000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -5000,17 +4765,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Рішення суду по кредиту — що робити далі</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>если есть решение суда по кредиту</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>18100000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>если есть решение суда по кредиту</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -5032,9 +4795,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5056,17 +4819,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -5089,17 +4852,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як виправити погану кредитну історію, якщо були прострочення</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как исправить кредитную историю если были просрочки</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>160000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -5118,17 +4879,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Чи впливає один день прострочки на кредитну історію</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>влияет ли один день просрочки на кредитную историю</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>436000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>влияет ли один день просрочки на кредитную историю</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -5147,17 +4906,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Чи впливає судова заборгованість на кредитну історію</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>влияет ли судебная задолженность на кредитную историю</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>761000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -5176,17 +4933,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Скільки зберігається кредитна історія в Україні</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>сколько хранится кредитная история в украине</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>10600000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -5205,17 +4960,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Через скільки «згоряє» кредитна історія</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>через сколько сгорает кредитная история</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>35700</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>срок исковой давности по кредиту в приватбанке</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -5234,17 +4987,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Чи дадуть кредит, якщо є прострочка по іншому кредиту</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>если есть просрочка по кредиту дадут ли кредит</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>31400</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -5263,17 +5014,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Чому мені не дають кредит: основні причини відмови</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>почему мне не дают кредит</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>2430000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -5292,17 +5041,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Через скільки часу кредит анулюється, якщо його не платити</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>если не платить кредит через сколько он аннулируется</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>22200</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -5321,17 +5068,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, чи є на мені кредити</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как узнать есть ли кредиты у меня</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>6250000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>исправлю кредитную историю</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -5350,17 +5095,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи може банк вимагати повернути весь кредит одразу</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>может ли банк потребовать вернуть весь кредит сразу</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>58</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -5379,17 +5122,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Чи має право банк збільшити відсоток за кредитом</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>имеет ли право банк увеличить процент по кредиту</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>2690000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>имеет ли право банк увеличить процент по кредиту</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -5408,17 +5149,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Як оскаржити комісію банку</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>как оспорить комиссию банка</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>61500000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>суд по ипотеке</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -5440,9 +5179,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5464,17 +5203,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -5497,17 +5236,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Чи можна виїхати з України, якщо є кредит</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>можно ли выехать из украины если есть кредит</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>808000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -5526,17 +5263,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Чи випустять за кордон з боргом по кредитній картці</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>1510</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -5555,17 +5290,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>З якою сумою боргу не випускають за кордон</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>с какой суммой задолженности не выпускают за границу</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>20400</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -5584,17 +5317,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як перевірити, чи є борги, перед виїздом за кордон</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как проверить есть ли долги для выезда за границу</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>60700</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -5613,17 +5344,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть колектори заборонити виїзд за кордон</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>могут ли коллекторы запретить выезд за границу</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>83</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -5642,17 +5371,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Чи випустять за кордон з іпотекою</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>выпустят ли за границу с ипотекой</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>198</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -5671,17 +5398,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися борги за прізвищем</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>как узнать долги по фамилии</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>458000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>проверка на долги по фио</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -5700,17 +5425,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися про всі свої борги по кредитах</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>как узнать все свои долги по кредитам</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>19800000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>проверка на долги по фио</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -5729,17 +5452,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть забрати пенсію за кредит</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>могут ли забрать пенсию за кредит</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>1390000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли забрать пенсию за кредит</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -5758,17 +5479,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Чи може інвалід 1 групи не платити кредит</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>может ли инвалид 1 группы не платить кредит</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>может ли инвалид 1 группы не платить кредит</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -5787,17 +5506,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Син узяв кредит і не платить: що робити батькам</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>сын взял кредит и не платит что делать</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>2070000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>сын взял кредит и не платит что делать</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -5816,17 +5533,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Що робити з кредитом, якщо людина у в’язниці</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>что делать с кредитом если человек в тюрьме</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>98</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что делать с кредитом если человек в тюрьме</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -5848,9 +5563,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5872,17 +5587,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -5905,17 +5620,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть звільнити з роботи за борги по кредитах</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>могут ли уволить за долги по кредитам</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>1010000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>просрочка по кредиту последствия</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -5934,17 +5647,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть забрати водійські права за несплату кредиту</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>могут ли забрать права за неуплату кредита</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>4410000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>просрочка по кредиту последствия</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -5963,17 +5674,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть позбавити батьківських прав за несплату кредиту</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>могут ли лишить родительских прав за неуплату кредита</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>15400</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли лишить родительских прав за неуплату кредита</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -5992,17 +5701,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть кредитори приїхати додому</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>могут ли кредиторы приехать домой</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>369000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли кредиторы приехать домой</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -6021,17 +5728,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Дружина набрала кредитів: що робити чоловіку</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>жена набрала кредитов что делать</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>76300</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>жена набрала кредитов что делать</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -6050,17 +5755,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Чи варто ховатися від кредиторів</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>как скрыться от кредиторов</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>6340000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как скрыться от кредиторов</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -6079,17 +5782,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Що роблять з боржниками по кредитах</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>что делают с должниками по кредитам</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>869000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что делают с должниками по кредитам</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -6108,17 +5809,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо зарплати не вистачає на кредити</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>что делать если зарплаты не хватает на кредиты</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>1850000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>что делать если зарплаты не хватает на кредиты</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -6137,17 +5836,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Втратив роботу — як платити кредит</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>если потерял работу как платить кредит</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>4420000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>если потерял работу как платить кредит</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -6166,17 +5863,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо взагалі не виплачувати кредит</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>если не выплачивать кредит</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>2480000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>если муж не платит кредит что грозит жене</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -6195,17 +5890,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Чи можна сплачувати кредит з-за кордону</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>можно ли оплачивать кредит из другой страны</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>4440000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>можно ли оплачивать кредит из другой страны</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -6224,17 +5917,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Чи може банк «забути» про кредит</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>может ли банк забыть про кредит</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>8180000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>может ли банк забыть про кредит</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -6256,9 +5947,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -6280,17 +5971,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -6313,17 +6004,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як визнати себе банкрутом фізичній особі</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>59800</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -6342,17 +6031,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо оголосити себе банкрутом: наслідки для фізособи</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>что если объявить себя банкротом</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>992000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -6371,17 +6058,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Що потрібно, щоб оголосити себе банкрутом: умови та документи</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>что надо чтобы объявить себя банкротом</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>1040000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -6400,17 +6085,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як колектори знаходять родичів боржника</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как коллекторы находят родственников</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>90</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -6429,17 +6112,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Як колектори дізнаються адресу боржника</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>как коллекторы узнают адрес</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>2410000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -6458,17 +6139,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Що буде, якщо не відповідати на дзвінки колекторів</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>что будет если не брать трубку от коллекторов</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>1080000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -6487,17 +6166,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Що можуть зробити колектори з родичами боржника</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>что могут сделать коллекторы родственникам должника</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>294000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -6516,17 +6193,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Як зупинити дзвінки колекторів</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>как остановить звонки коллекторов</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>120000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -6545,17 +6220,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть колектори продати борг іншим колекторам</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>могут ли коллекторы продать долг другим коллекторам</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>24000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>заказное письмо от мфо</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -6574,17 +6247,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Дзвінки колекторів за чужим кредитом — як позбутися</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>как избавиться от звонков коллекторов по чужому кредиту</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>28400</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как избавиться от звонков коллекторов по чужому кредиту</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -6603,17 +6274,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Хто такий антиколектор і чим він допомагає</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>кто такой антиколлектор</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>23900</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>отзывы о коллекторах</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -6632,17 +6301,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Як розмовляти з колекторами, якщо немає грошей</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>как разговаривать с коллекторами если нет денег</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>43400</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>заказное письмо от мфо</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -6664,9 +6331,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -6688,17 +6355,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -6721,17 +6388,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як списати борги по кредитній картці</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как списать долги по кредитной карте</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>95400</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -6750,17 +6415,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Як законно списати кредити</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>как законно списать кредиты</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>130000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -6779,17 +6442,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Коли спишуть кредити</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>когда спишут кредиты</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>5950000</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>приватбанк списание долгов</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -6808,17 +6469,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть МФО відібрати квартиру за борги</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>могут ли мфо отобрать квартиру</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>272000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>могут ли мфо отобрать квартиру</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -6837,17 +6496,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Чи може МФО подати заяву в поліцію на боржника</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>может ли мфо подать заявление в полицию</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>1520000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>может ли мфо подать заявление в полицию</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -6866,17 +6523,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Чи спишуть борги по кредитах пенсіонерам</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>спишут ли долги по кредитам пенсионерам</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>1360000</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>спишут ли долги по кредитам пенсионерам</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -6895,17 +6550,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Які кредити списують</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>какие кредиты списывают</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>2750000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>какие кредиты списывают</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -6924,17 +6577,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть МФО пробачити борг</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>могут ли мфо простить долг</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>24800</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как списать долги по мфо</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -6953,17 +6604,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Як позбутися кредитних боргів законно</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>как избавиться от кредитных долгов законно</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>112000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -6982,17 +6631,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Як списати відсотки по мікрозайму</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>как списать проценты по микрозайму</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>7920</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -7011,17 +6658,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, чи списали мені кредит</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>как узнать списали ли мне кредит</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>713000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -7040,17 +6685,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Куди звернутися, щоб списали кредит</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>куда обратится чтобы списали кредит</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>300000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как списать долги по мфо</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -7072,9 +6715,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -7096,17 +6739,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Фокусна фраза (питання)</t>
+          <t>Фокусна фраза (ключ із семантики)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Вихідний ключ із семантики</t>
+          <t>Частотність</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Тип статті</t>
+          <t>Кластер</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -7129,17 +6772,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Як дізнатися, чи взято на мене мікрозайм</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>как узнать взят ли на меня микрозайм</t>
         </is>
       </c>
+      <c r="E2" s="3" t="n">
+        <v>1520000</v>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -7158,17 +6799,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо на вас оформили мікрозайм</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>что делать если на тебя оформили микрозайм</t>
         </is>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>27900000</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -7187,17 +6826,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Чи можуть оформити кредит без мого відома</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>могут ли оформить кредит без моего ведома</t>
         </is>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>200</v>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -7216,17 +6853,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Як захиститися від кредитних шахраїв</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
           <t>как защититься от кредитных мошенников</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>2290000</v>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -7245,17 +6880,15 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо шахраї змусили взяти кредит</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>что делать если мошенники заставили взять кредит</t>
         </is>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>200000</v>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -7274,17 +6907,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Як довести, що ти не брав кредит</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
           <t>как доказать что ты не брал кредит</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>100</v>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -7303,17 +6934,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Як оскаржити кредит, який ви не брали</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>как оспорить кредит который не брал</t>
         </is>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>1170000</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -7332,17 +6961,15 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Телефонують і кажуть, що на вас оформлено кредит: що це</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
           <t>звонят говорят что на вас оформлен кредит</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>6590000</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -7361,17 +6988,15 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Чи безпечно брати позику через інтернет</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>безопасно ли брать займ через интернет</t>
         </is>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>71800000</v>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -7390,17 +7015,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Куди звертатися, якщо на мене оформили кредит</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
           <t>куда обращаться если на меня оформили кредит</t>
         </is>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>8620000</v>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -7419,17 +7042,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Як визнати договір з МФО недійсним</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>как признать договор с мфо недействительным</t>
         </is>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>118000</v>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>оспаривание кредитного договора</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -7448,17 +7069,15 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Що робити, якщо втратили кредитний договір</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>что делать если потерял кредитный договор</t>
         </is>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>3390000</v>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Розбір питання</t>
+          <t>оспаривание кредитного договора</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add copywriting style cards and Style column for 16 sites
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,7 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -489,6 +490,11 @@
           <t>Статей</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Манера стилю (джерело)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -517,6 +523,11 @@
       <c r="F2" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Манера підручника цивільного права (за ТЗ: Борисова та ін.). Якір: «X — це …» (див. ТЗ)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -545,6 +556,11 @@
       <c r="F3" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Банківське право: нормативний виклад (Лаврик, Терела, за ТЗ)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -573,6 +589,11 @@
       <c r="F4" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Огляд практики Верховного Суду: позиція → що це означає → «Детальніше…» (за ТЗ)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -601,6 +622,11 @@
       <c r="F5" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Сімейне право: «по-перше / по-друге», норма → виняток (Апопій, за ТЗ)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -629,6 +655,11 @@
       <c r="F6" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Кримінальний процес і правнича допомога: нумеровані групи 1) 2) 3) (Тертишник, за ТЗ)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -657,6 +688,11 @@
       <c r="F7" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Аналітична записка: проблема → практика судів → «Отже, є підстави вважати …» → рекомендації (Григорян, PRAVO-Justice)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -685,6 +721,11 @@
       <c r="F8" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Концептуальний академізм: «Слід наголосити …», «До цього додамо …» (Кучерявенко, Фінансове право, 2019)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -713,6 +754,11 @@
       <c r="F9" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Консультаційний алгоритм: кроки, тест-питання, «Ви» (Порадник клініциста, ЧНУ)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -741,6 +787,11 @@
       <c r="F10" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Суддівське есе: нумеровані міркування, «Тож …», «Втім …» (Крат, «Трохи про право іпотеки», 2024)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -769,6 +820,11 @@
       <c r="F11" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Медіаційний гуманістичний тон: інтереси сторін, гнучка процедура (Крестовська, Романадзе, «Медіація у професійній діяльності юриста», 2019)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -797,6 +853,11 @@
       <c r="F12" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Процедурний довідник: визначення зі ст. закону, переліки реквізитів (Білоусов, «Виконавче провадження»)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -825,6 +886,11 @@
       <c r="F13" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Ситуаційні завдання: ситуація → питання → відповідь (Практикум з цивільного процесуального права, КНЕУ)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -853,6 +919,11 @@
       <c r="F14" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Практикум-тест: «Перевірте себе», питання з варіантами а) б) в) (Тодорошко, «Цивільно-процесуальне право: практикум»)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -881,6 +952,11 @@
       <c r="F15" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Позовна аргументація: «Щодо …», нумерація 1., 1.1., «у нашому випадку» (посібник КМА «Юридичні клініки на захисті прав споживачів фінансових послуг», 2020)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -909,6 +985,11 @@
       <c r="F16" s="2" t="n">
         <v>12</v>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Договірне право: поняття → сторони → предмет → форма → зміст (Кириченко, Кириченко, Куракін, 2024)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -936,6 +1017,11 @@
       </c>
       <c r="F17" s="2" t="n">
         <v>12</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Нормативно-пояснювальний виклад: «Відповідно до …», «Отже, підставами є …» (Бехруз, Мануїлова, «Фінансове право», 2022)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -949,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -959,6 +1045,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -997,6 +1084,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1024,6 +1116,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1051,6 +1148,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1078,6 +1180,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1105,6 +1212,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1132,6 +1244,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1159,6 +1276,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1186,6 +1308,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1213,6 +1340,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1240,6 +1372,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1267,6 +1404,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1294,6 +1436,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1321,6 +1468,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1333,7 +1485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1343,6 +1495,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1381,6 +1534,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1408,6 +1566,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1435,6 +1598,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1462,6 +1630,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1489,6 +1662,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1516,6 +1694,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1543,6 +1726,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1570,6 +1758,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1597,6 +1790,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1624,6 +1822,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1651,6 +1854,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1678,6 +1886,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1705,6 +1918,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1717,7 +1935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1727,6 +1945,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1765,6 +1984,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1792,6 +2016,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1819,6 +2048,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1846,6 +2080,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1873,6 +2112,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1900,6 +2144,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1927,6 +2176,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1954,6 +2208,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1981,6 +2240,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2008,6 +2272,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2035,6 +2304,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2062,6 +2336,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2089,6 +2368,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2101,7 +2385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2111,6 +2395,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2149,6 +2434,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2176,6 +2466,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2203,6 +2498,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2230,6 +2530,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2257,6 +2562,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2284,6 +2594,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2311,6 +2626,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2338,6 +2658,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2365,6 +2690,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2392,6 +2722,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2419,6 +2754,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2446,6 +2786,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2473,6 +2818,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2485,7 +2835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2495,6 +2845,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2533,6 +2884,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2560,6 +2916,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2587,6 +2948,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2614,6 +2980,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2641,6 +3012,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2668,6 +3044,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2695,6 +3076,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2722,6 +3108,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2749,6 +3140,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2776,6 +3172,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2803,6 +3204,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2830,6 +3236,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2857,6 +3268,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2869,7 +3285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2879,6 +3295,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2917,6 +3334,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2944,6 +3366,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2971,6 +3398,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2998,6 +3430,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3025,6 +3462,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3052,6 +3494,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3079,6 +3526,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3106,6 +3558,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3133,6 +3590,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3160,6 +3622,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3187,6 +3654,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3214,6 +3686,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3241,6 +3718,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3253,7 +3735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3263,6 +3745,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3301,6 +3784,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -3328,6 +3816,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -3355,6 +3848,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3382,6 +3880,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3409,6 +3912,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3436,6 +3944,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3463,6 +3976,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3490,6 +4008,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3517,6 +4040,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3544,6 +4072,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3571,6 +4104,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3598,6 +4136,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3625,6 +4168,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3637,7 +4185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3647,6 +4195,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3685,6 +4234,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -3712,6 +4266,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -3739,6 +4298,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3766,6 +4330,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3793,6 +4362,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3820,6 +4394,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3847,6 +4426,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3874,6 +4458,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3901,6 +4490,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3928,6 +4522,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3955,6 +4554,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3982,6 +4586,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -4009,6 +4618,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4021,7 +4635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4031,6 +4645,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4069,6 +4684,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4096,6 +4716,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4123,6 +4748,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4150,6 +4780,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4177,6 +4812,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4204,6 +4844,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4231,6 +4876,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4258,6 +4908,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4285,6 +4940,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4312,6 +4972,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4339,6 +5004,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -4366,6 +5036,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -4393,6 +5068,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4405,7 +5085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4415,6 +5095,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4453,6 +5134,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4480,6 +5166,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4507,6 +5198,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4534,6 +5230,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4561,6 +5262,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4588,6 +5294,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4615,6 +5326,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4642,6 +5358,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4669,6 +5390,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4696,6 +5422,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4723,6 +5454,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -4750,6 +5486,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -4777,6 +5518,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4789,7 +5535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4799,6 +5545,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4837,6 +5584,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4864,6 +5616,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4891,6 +5648,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4918,6 +5680,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4945,6 +5712,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4972,6 +5744,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4999,6 +5776,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -5026,6 +5808,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -5053,6 +5840,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -5080,6 +5872,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -5107,6 +5904,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -5134,6 +5936,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -5161,6 +5968,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5173,7 +5985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5183,6 +5995,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5221,6 +6034,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -5248,6 +6066,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -5275,6 +6098,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -5302,6 +6130,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -5329,6 +6162,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -5356,6 +6194,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -5383,6 +6226,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -5410,6 +6258,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -5437,6 +6290,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -5464,6 +6322,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -5491,6 +6354,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -5518,6 +6386,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -5545,6 +6418,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5557,7 +6435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5567,6 +6445,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5605,6 +6484,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -5632,6 +6516,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -5659,6 +6548,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -5686,6 +6580,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -5713,6 +6612,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -5740,6 +6644,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -5767,6 +6676,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -5794,6 +6708,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -5821,6 +6740,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -5848,6 +6772,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -5875,6 +6804,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -5902,6 +6836,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -5929,6 +6868,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5941,7 +6885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5951,6 +6895,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5989,6 +6934,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -6016,6 +6966,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -6043,6 +6998,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -6070,6 +7030,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -6097,6 +7062,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -6124,6 +7094,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -6151,6 +7126,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -6178,6 +7158,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -6205,6 +7190,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -6232,6 +7222,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -6259,6 +7254,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -6286,6 +7286,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -6313,6 +7318,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6325,7 +7335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6335,6 +7345,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6373,6 +7384,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -6400,6 +7416,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -6427,6 +7448,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -6454,6 +7480,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -6481,6 +7512,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -6508,6 +7544,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -6535,6 +7576,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -6562,6 +7608,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -6589,6 +7640,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -6616,6 +7672,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -6643,6 +7704,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -6670,6 +7736,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -6697,6 +7768,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6709,7 +7785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6719,6 +7795,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6757,6 +7834,11 @@
           <t>Статус ТЗ</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -6784,6 +7866,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -6811,6 +7898,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -6838,6 +7930,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -6865,6 +7962,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -6892,6 +7994,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -6919,6 +8026,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -6946,6 +8058,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -6973,6 +8090,11 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -7000,6 +8122,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -7027,6 +8154,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -7054,6 +8186,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -7081,6 +8218,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Content plans: focus phrases translated to Ukrainian
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как попросить у банка отсрочку по кредиту</t>
+          <t>як попросити в банку відстрочку за кредитом</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>как получить кредитные каникулы в банке</t>
+          <t>як отримати кредитні канікули в банку</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>как оформить кредитные каникулы в мфо</t>
+          <t>як оформити кредитні канікули в МФО</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как написать письмо в банк об отсрочке платежа</t>
+          <t>як написати лист у банк про відстрочку платежу</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как снизить ставку по кредиту</t>
+          <t>як знизити ставку за кредитом</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>как договориться с мфо о рассрочке</t>
+          <t>як домовитися з МФО про розстрочку</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>как договориться с мфо о списании процентов</t>
+          <t>як домовитися з МФО про списання відсотків</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>как оплатить только тело кредита мфо</t>
+          <t>як сплатити лише тіло кредиту МФО</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как закрыть микрозайм если нет денег</t>
+          <t>як закрити мікрозайм якщо немає грошей</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>можно ли платить микрозайм частями</t>
+          <t>чи можна платити мікрозайм частинами</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>как лучше закрыть кредит досрочно</t>
+          <t>як краще закрити кредит достроково</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>что значит заморозить займ</t>
+          <t>що означає заморозити позику</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как узнать есть ли ты в реестре должников</t>
+          <t>як дізнатися чи є ти в реєстрі боржників</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>как убрать себя с реестра должников</t>
+          <t>як прибрати себе з реєстру боржників</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>если висит долг у судебных приставов</t>
+          <t>якщо висить борг у судових приставів</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>могут ли арестовать счета без суда</t>
+          <t>чи можуть заарештувати рахунки без суду</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>какие выплаты не подлежат аресту</t>
+          <t>які виплати не підлягають арешту</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>на какие счета нельзя накладывать арест</t>
+          <t>на які рахунки не можна накладати арешт</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>можно ли пользоваться картой если на ней арест</t>
+          <t>чи можна користуватися карткою якщо на ній арешт</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>как получать зарплату если карта арестована</t>
+          <t>як отримувати зарплату якщо картку арештовано</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>можно ли снять арест с зарплатной карты</t>
+          <t>чи можна зняти арешт із зарплатної картки</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>как узнать арестован счет или нет</t>
+          <t>як дізнатися чи арештовано рахунок</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>имеют ли право наложить арест на детское пособие</t>
+          <t>чи мають право накласти арешт на дитячу допомогу</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>через сколько снимается арест с карты после оплаты</t>
+          <t>через скільки знімається арешт з картки після оплати</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как отменить решение суда по кредиту</t>
+          <t>як скасувати рішення суду за кредитом</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>апелляция на решение суда по кредиту</t>
+          <t>апеляція на рішення суду за кредитом</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>что такое срок исковой давности по кредиту</t>
+          <t>що таке строк позовної давності за кредитом</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как бороться с приватбанком</t>
+          <t>як боротися з ПриватБанком</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как узнать кто подал в суд по кредиту</t>
+          <t>як дізнатися хто подав до суду за кредитом</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>повестка в суд за неуплату кредита</t>
+          <t>повістка до суду за несплату кредиту</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>чем грозит суд по кредиту</t>
+          <t>чим загрожує суд за кредитом</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>почему банк не подает в суд по кредиту</t>
+          <t>чому банк не подає до суду за кредитом</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>что говорить в суде по кредиту</t>
+          <t>що говорити в суді за кредитом</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>можно ли выиграть суд с банком</t>
+          <t>чи можна виграти суд з банком</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>как оспорить проценты по кредиту в суде</t>
+          <t>як оскаржити відсотки за кредитом у суді</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>может ли суд отменить проценты по кредиту</t>
+          <t>чи може суд скасувати відсотки за кредитом</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>банк обратился в суд что делать</t>
+          <t>банк звернувся до суду що робити</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>как вести себя в суде с банком</t>
+          <t>як поводитися в суді з банком</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>как оспорить решение суда по микрозаймам</t>
+          <t>як оскаржити рішення суду по мікрозаймах</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как выиграть суд у микрофинансовой организации</t>
+          <t>як виграти суд у мікрофінансової організації</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как подать иск в суд на мфо</t>
+          <t>як подати позов до суду на МФО</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>можно ли подать в суд на банк</t>
+          <t>чи можна подати до суду на банк</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>как судиться с мфо</t>
+          <t>як судитися з МФО</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>если мфо подала в суд</t>
+          <t>якщо МФО подала до суду</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>через какое время мфо подает в суд</t>
+          <t>через який час МФО подає до суду</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>как снизить проценты по микрозайму в суде</t>
+          <t>як знизити відсотки по мікрозайму в суді</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>начисляются ли проценты по кредиту после решения суда</t>
+          <t>чи нараховуються відсотки за кредитом після рішення суду</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>кто судился с приватбанком</t>
+          <t>хто судився з ПриватБанком</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>что делать если не можешь выплатить займ</t>
+          <t>що робити якщо не можеш виплатити позику</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>как вести себя с мфо при просрочке</t>
+          <t>як поводитися з МФО при простроченні</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>куча долгов в мфо что делать</t>
+          <t>купа боргів у МФО що робити</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>что делать если много займов</t>
+          <t>що робити якщо багато позик</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>если долги в нескольких банках</t>
+          <t>якщо борги в кількох банках</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>кто может помочь с долгами</t>
+          <t>хто може допомогти з боргами</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>что такое микрокредитование и чем оно опасно</t>
+          <t>що таке мікрокредитування і чим воно небезпечне</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>большой долг в микрозайме что делать</t>
+          <t>великий борг у мікрозаймі що робити</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>сколько максимум процентов может начислить мфо</t>
+          <t>скільки максимум відсотків може нарахувати МФО</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>может ли пеня превышать сумму долга</t>
+          <t>чи може пеня перевищувати суму боргу</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>могут ли проценты превышать сумму займа</t>
+          <t>чи можуть відсотки перевищувати суму позики</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>как посчитать процент просрочки по кредиту</t>
+          <t>як порахувати відсоток прострочення за кредитом</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как сделать реструктуризацию кредита в приватбанке</t>
+          <t>як зробити реструктуризацію кредиту в ПриватБанку</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>долг в приватбанке что делать</t>
+          <t>борг у ПриватБанку що робити</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>как узнать есть ли долг в приватбанке</t>
+          <t>як дізнатися чи є борг у ПриватБанку</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как погасить кредит в приватбанке если нет денег</t>
+          <t>як погасити кредит у ПриватБанку якщо немає грошей</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как начисляются проценты по кредитной карте приватбанка</t>
+          <t>як нараховуються відсотки по кредитній картці ПриватБанку</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>что будет если не оплачивать кредитную карту</t>
+          <t>що буде якщо не сплачувати кредитну картку</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>может ли приват банк списать долг</t>
+          <t>чи може ПриватБанк списати борг</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>как рассчитать обязательный платеж по кредитной карте приватбанка</t>
+          <t>як розрахувати обов'язковий платіж по кредитній картці ПриватБанку</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как правильно закрыть кредитку приватбанка</t>
+          <t>як правильно закрити кредитку ПриватБанку</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>что значит пролонгация кредита</t>
+          <t>що означає пролонгація кредиту</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>можно ли расторгнуть кредитный договор с банком</t>
+          <t>чи можна розірвати кредитний договір з банком</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>если у банка нет оригинала кредитного договора</t>
+          <t>якщо в банку немає оригіналу кредитного договору</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>переплатила кредит что делать</t>
+          <t>переплатила за кредитом що робити</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>как вернуть часть денег за кредит</t>
+          <t>як повернути частину грошей за кредит</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>нужно ли идти в банк после погашения кредита</t>
+          <t>чи потрібно йти в банк після погашення кредиту</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>нужно ли писать заявление на досрочное погашение кредита</t>
+          <t>чи потрібно писати заяву на дострокове погашення кредиту</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как погасить кредит если карта заблокирована</t>
+          <t>як погасити кредит якщо картку заблоковано</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>можно ли погасить кредит и сразу взять новый</t>
+          <t>чи можна погасити кредит і одразу взяти новий</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>что делать если срок действия кредитной карты истек</t>
+          <t>що робити якщо строк дії кредитної картки закінчився</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>можно ли погасить кредит через месяц</t>
+          <t>чи можна погасити кредит через місяць</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>что будет если не платить кредит за телефон</t>
+          <t>що буде якщо не платити кредит за телефон</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>может ли банк списать долг по кредиту с зарплатной карты</t>
+          <t>чи може банк списати борг за кредитом із зарплатної картки</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>какие документы нужны для закрытия кредита</t>
+          <t>які документи потрібні для закриття кредиту</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -4606,7 +4606,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>как взять справку о закрытии кредита</t>
+          <t>як взяти довідку про закриття кредиту</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>что будет за просрочку кредита</t>
+          <t>що буде за прострочення кредиту</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>могут ли за долги посадить</t>
+          <t>чи можуть за борги посадити</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>как оспорить кредитный договор с банком</t>
+          <t>як оскаржити кредитний договір з банком</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>банк передал дело коллекторам что делать</t>
+          <t>банк передав справу колекторам що робити</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>могут ли заблокировать кредитную карту приставы</t>
+          <t>чи можуть заблокувати кредитну картку пристави</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>как уменьшить сумму платежа по кредиту</t>
+          <t>як зменшити суму платежу за кредитом</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>можно ли не платить кредит если прошло 3 года</t>
+          <t>чи можна не платити кредит якщо минуло 3 роки</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>пришел судебный приказ о взыскании задолженности по кредиту</t>
+          <t>прийшов судовий наказ про стягнення заборгованості за кредитом</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как реструктуризировать микрозаймы</t>
+          <t>як реструктуризувати мікрозайми</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>могут ли коллекторы наложить арест на имущество</t>
+          <t>чи можуть колектори накласти арешт на майно</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>если муж не платит кредит что грозит жене</t>
+          <t>якщо чоловік не платить кредит що загрожує дружині</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>что будет если не платить кредит под залог недвижимости</t>
+          <t>що буде якщо не платити кредит під заставу нерухомості</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>что будет если не платить по исполнительному листу</t>
+          <t>що буде якщо не платити за виконавчим листом</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>можно ли договориться с приставами</t>
+          <t>чи можна домовитися з приставами</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>что делать если пришел исполнительный лист по кредиту</t>
+          <t>що робити якщо прийшов виконавчий лист за кредитом</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как уменьшить выплаты по исполнительному листу</t>
+          <t>як зменшити виплати за виконавчим листом</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как отменить исполнительное производство по кредиту</t>
+          <t>як скасувати виконавче провадження за кредитом</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>как прекратить исполнительное производство если долг погашен</t>
+          <t>як припинити виконавче провадження якщо борг погашено</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>можно ли отменить исполнительный лист</t>
+          <t>чи можна скасувати виконавчий лист</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>как закрыть задолженность у судебных приставов</t>
+          <t>як закрити заборгованість у приставів</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как не платить долг по решению суда</t>
+          <t>як не платити борг за рішенням суду</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>могут ли приставы снимать все деньги с зарплатной карты</t>
+          <t>чи можуть пристави знімати всі гроші із зарплатної картки</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>что делать с исполнительным листом</t>
+          <t>що робити з виконавчим листом</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>если есть решение суда по кредиту</t>
+          <t>якщо є рішення суду за кредитом</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как исправить кредитную историю если были просрочки</t>
+          <t>як виправити кредитну історію якщо були прострочення</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>влияет ли один день просрочки на кредитную историю</t>
+          <t>чи впливає один день прострочення на кредитну історію</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>влияет ли судебная задолженность на кредитную историю</t>
+          <t>чи впливає судова заборгованість на кредитну історію</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>сколько хранится кредитная история в украине</t>
+          <t>скільки зберігається кредитна історія в Україні</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>через сколько сгорает кредитная история</t>
+          <t>через скільки згорає кредитна історія</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>если есть просрочка по кредиту дадут ли кредит</t>
+          <t>якщо є прострочення за кредитом чи дадуть кредит</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>почему мне не дают кредит</t>
+          <t>чому мені не дають кредит</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -5828,7 +5828,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>если не платить кредит через сколько он аннулируется</t>
+          <t>якщо не платити кредит через скільки він анулюється</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как узнать есть ли кредиты у меня</t>
+          <t>як дізнатися чи є в мене кредити</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>может ли банк потребовать вернуть весь кредит сразу</t>
+          <t>чи може банк вимагати повернути весь кредит одразу</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>имеет ли право банк увеличить процент по кредиту</t>
+          <t>чи має право банк збільшити відсоток за кредитом</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>как оспорить комиссию банка</t>
+          <t>як оскаржити комісію банку</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>можно ли выехать из украины если есть кредит</t>
+          <t>чи можна виїхати з України якщо є кредит</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>выпустят ли за границу с долгом по кредитной карте</t>
+          <t>чи випустять за кордон з боргом по кредитній картці</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -6118,7 +6118,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>с какой суммой задолженности не выпускают за границу</t>
+          <t>з якою сумою заборгованості не випускають за кордон</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как проверить есть ли долги для выезда за границу</t>
+          <t>як перевірити чи є борги для виїзду за кордон</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>могут ли коллекторы запретить выезд за границу</t>
+          <t>чи можуть колектори заборонити виїзд за кордон</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>выпустят ли за границу с ипотекой</t>
+          <t>чи випустять за кордон з іпотекою</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -6246,7 +6246,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>как узнать долги по фамилии</t>
+          <t>як дізнатися борги за прізвищем</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>как узнать все свои долги по кредитам</t>
+          <t>як дізнатися всі свої борги по кредитах</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>могут ли забрать пенсию за кредит</t>
+          <t>чи можуть забрати пенсію за кредит</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>может ли инвалид 1 группы не платить кредит</t>
+          <t>чи може інвалід 1 групи не платити кредит</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>сын взял кредит и не платит что делать</t>
+          <t>син узяв кредит і не платить що робити</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>что делать с кредитом если человек в тюрьме</t>
+          <t>що робити з кредитом якщо людина у в'язниці</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -6504,7 +6504,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>могут ли уволить за долги по кредитам</t>
+          <t>чи можуть звільнити за борги по кредитах</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>могут ли забрать права за неуплату кредита</t>
+          <t>чи можуть забрати права за несплату кредиту</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>могут ли лишить родительских прав за неуплату кредита</t>
+          <t>чи можуть позбавити батьківських прав за несплату кредиту</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -6600,7 +6600,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>могут ли кредиторы приехать домой</t>
+          <t>чи можуть кредитори приїхати додому</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>жена набрала кредитов что делать</t>
+          <t>дружина набрала кредитів що робити</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>как скрыться от кредиторов</t>
+          <t>як сховатися від кредиторів</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>что делают с должниками по кредитам</t>
+          <t>що роблять з боржниками по кредитах</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>что делать если зарплаты не хватает на кредиты</t>
+          <t>що робити якщо зарплати не вистачає на кредити</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>если потерял работу как платить кредит</t>
+          <t>якщо втратив роботу як платити кредит</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>если не выплачивать кредит</t>
+          <t>якщо не виплачувати кредит</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>можно ли оплачивать кредит из другой страны</t>
+          <t>чи можна сплачувати кредит з-за кордону</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>может ли банк забыть про кредит</t>
+          <t>чи може банк забути про кредит</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как признать себя банкротом физ лицо</t>
+          <t>як визнати себе банкрутом фізична особа</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -6986,7 +6986,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>что если объявить себя банкротом</t>
+          <t>що якщо оголосити себе банкрутом</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>что надо чтобы объявить себя банкротом</t>
+          <t>що потрібно щоб оголосити себе банкрутом</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как коллекторы находят родственников</t>
+          <t>як колектори знаходять родичів</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>как коллекторы узнают адрес</t>
+          <t>як колектори дізнаються адресу</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>что будет если не брать трубку от коллекторов</t>
+          <t>що буде якщо не брати слухавку від колекторів</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>что могут сделать коллекторы родственникам должника</t>
+          <t>що можуть зробити колектори родичам боржника</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>как остановить звонки коллекторов</t>
+          <t>як зупинити дзвінки колекторів</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>могут ли коллекторы продать долг другим коллекторам</t>
+          <t>чи можуть колектори продати борг іншим колекторам</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>как избавиться от звонков коллекторов по чужому кредиту</t>
+          <t>як позбутися дзвінків колекторів за чужим кредитом</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>кто такой антиколлектор</t>
+          <t>хто такий антиколектор</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -7306,7 +7306,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>как разговаривать с коллекторами если нет денег</t>
+          <t>як розмовляти з колекторами якщо немає грошей</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как списать долги по кредитной карте</t>
+          <t>як списати борги по кредитній картці</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>как законно списать кредиты</t>
+          <t>як законно списати кредити</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>когда спишут кредиты</t>
+          <t>коли спишуть кредити</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -7500,7 +7500,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>могут ли мфо отобрать квартиру</t>
+          <t>чи можуть МФО забрати квартиру</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>может ли мфо подать заявление в полицию</t>
+          <t>чи може МФО подати заяву в поліцію</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>спишут ли долги по кредитам пенсионерам</t>
+          <t>чи спишуть борги по кредитах пенсіонерам</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>какие кредиты списывают</t>
+          <t>які кредити списують</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>могут ли мфо простить долг</t>
+          <t>чи можуть МФО пробачити борг</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как избавиться от кредитных долгов законно</t>
+          <t>як позбутися кредитних боргів законно</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>как списать проценты по микрозайму</t>
+          <t>як списати відсотки по мікрозайму</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>как узнать списали ли мне кредит</t>
+          <t>як дізнатися чи списали мені кредит</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>куда обратится чтобы списали кредит</t>
+          <t>куди звернутися щоб списали кредит</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>как узнать взят ли на меня микрозайм</t>
+          <t>як дізнатися чи взято на мене мікрозайм</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>что делать если на тебя оформили микрозайм</t>
+          <t>що робити якщо на тебе оформили мікрозайм</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>могут ли оформить кредит без моего ведома</t>
+          <t>чи можуть оформити кредит без мого відома</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как защититься от кредитных мошенников</t>
+          <t>як захиститися від кредитних шахраїв</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>что делать если мошенники заставили взять кредит</t>
+          <t>що робити якщо шахраї змусили взяти кредит</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>как доказать что ты не брал кредит</t>
+          <t>як довести що ти не брав кредит</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -8046,7 +8046,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>как оспорить кредит который не брал</t>
+          <t>як оскаржити кредит який не брав</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>звонят говорят что на вас оформлен кредит</t>
+          <t>дзвонять кажуть що на вас оформлено кредит</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>безопасно ли брать займ через интернет</t>
+          <t>чи безпечно брати позику через інтернет</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -8142,7 +8142,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>куда обращаться если на меня оформили кредит</t>
+          <t>куди звертатися якщо на мене оформили кредит</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>как признать договор с мфо недействительным</t>
+          <t>як визнати договір з МФО недійсним</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>что делать если потерял кредитный договор</t>
+          <t>що робити якщо втратив кредитний договір</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">

</xml_diff>

<commit_message>
Content plans xlsx: Ukrainian phrases for mortgage site tab
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -1104,7 +1104,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>чем опасен кредит под залог квартиры</t>
+          <t>чим небезпечний кредит під заставу квартири</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>можно ли купить квартиру если есть долги по кредитам</t>
+          <t>чи можна купити квартиру якщо є борги по кредитах</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>можно ли продать квартиру если есть долги по кредитам</t>
+          <t>чи можна продати квартиру якщо є борги по кредитах</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>как взять отсрочку по ипотеке</t>
+          <t>як взяти відстрочку по іпотеці</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>плохая кредитная история как взять ипотеку</t>
+          <t>погана кредитна історія як взяти іпотеку</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>как узнать снят ли арест с квартиры</t>
+          <t>як дізнатися чи знято арешт з квартири</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>как снять арест с автомобиля наложенный судом</t>
+          <t>як зняти арешт з автомобіля накладений судом</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>можно ли продать авто которое в кредите</t>
+          <t>чи можна продати авто яке в кредиті</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>как проверить наложен ли арест на квартиру</t>
+          <t>як перевірити чи накладено арешт на квартиру</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>как снять залог с авто после погашения кредита</t>
+          <t>як зняти заставу з авто після погашення кредиту</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>что делать если на машину наложен арест</t>
+          <t>що робити якщо на машину накладено арешт</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>как вернуть кредитный автомобиль банку</t>
+          <t>як повернути кредитний автомобіль банку</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">

</xml_diff>

<commit_message>
Content plans: add cluster frequency column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1044,8 +1044,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1081,10 +1082,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -1115,8 +1121,11 @@
           <t>чем опасен кредит под залог квартиры</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>828000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1147,8 +1156,11 @@
           <t>можно ли купить квартиру если есть долги по кредитам</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>121000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1179,8 +1191,11 @@
           <t>можно ли продать квартиру если есть долги по кредитам</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>17700000</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1211,8 +1226,11 @@
           <t>что значит заморозить займ</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>56600</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1243,8 +1261,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1275,8 +1296,11 @@
           <t>как проверить арест на движимое имущество</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>53300</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1307,8 +1331,11 @@
           <t>как вернуть кредитную машину</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>1080000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1339,8 +1366,11 @@
           <t>можно ли обменять кредитную машину на другую</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>1310000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1371,8 +1401,11 @@
           <t>как проверить арест на движимое имущество</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>53300</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1403,8 +1436,11 @@
           <t>как вернуть кредитную машину</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>1080000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1435,8 +1471,11 @@
           <t>как вернуть кредитную машину</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>1080000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1467,8 +1506,11 @@
           <t>как вернуть кредитный автомобиль банку</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>7710000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1485,7 +1527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1494,8 +1536,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1531,10 +1574,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -1565,8 +1613,11 @@
           <t>что значит заморозить займ</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>56600</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1597,8 +1648,11 @@
           <t>что значит заморозить займ</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>56600</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1629,8 +1683,11 @@
           <t>что значит заморозить займ</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>56600</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1661,8 +1718,11 @@
           <t>что значит заморозить займ</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>56600</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1693,8 +1753,11 @@
           <t>как снизить ставку по кредиту</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>6710000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1725,8 +1788,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1757,8 +1823,11 @@
           <t>помощь в закрытии долгов</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1789,8 +1858,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1821,8 +1893,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1853,8 +1928,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1885,8 +1963,11 @@
           <t>как лучше закрыть кредит досрочно</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>656000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1917,8 +1998,11 @@
           <t>что значит заморозить займ</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>56600</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -1935,7 +2019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1944,8 +2028,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1981,10 +2066,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -2015,8 +2105,11 @@
           <t>как убрать себя с реестра должников</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>226000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2047,8 +2140,11 @@
           <t>как убрать себя с реестра должников</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>226000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2079,8 +2175,11 @@
           <t>если висит долг у судебных приставов</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2111,8 +2210,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2143,8 +2245,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2175,8 +2280,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2207,8 +2315,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2239,8 +2350,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2271,8 +2385,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2303,8 +2420,11 @@
           <t>как проверить арест на движимое имущество</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>53300</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2335,8 +2455,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2367,8 +2490,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2385,7 +2511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2394,8 +2520,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2431,10 +2558,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -2465,8 +2597,11 @@
           <t>как отменить решение суда по кредиту</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>3590000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2497,8 +2632,11 @@
           <t>апелляция на решение суда по кредиту</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2529,8 +2667,11 @@
           <t>срок исковой давности по кредиту в приватбанке</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>1790</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2561,8 +2702,11 @@
           <t>суд с приватбанком и как разорвать договор по кредитке</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2593,8 +2737,11 @@
           <t>как узнать кто подал в суд по кредиту</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2625,8 +2772,11 @@
           <t>повестка в суд за неуплату кредита</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>122000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2657,8 +2807,11 @@
           <t>просрочка по кредиту последствия</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>461000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2689,8 +2842,11 @@
           <t>почему банк не подает в суд по кредиту</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>14400000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2721,8 +2877,11 @@
           <t>суд по ипотеке</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2753,8 +2912,11 @@
           <t>суд по ипотеке</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2785,8 +2947,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2817,8 +2982,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2835,7 +3003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2844,8 +3012,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2881,10 +3050,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -2915,8 +3089,11 @@
           <t>суд по ипотеке</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2947,8 +3124,11 @@
           <t>суд по ипотеке</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -2979,8 +3159,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3011,8 +3194,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3043,8 +3229,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3075,8 +3264,11 @@
           <t>суд по ипотеке</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3107,8 +3299,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3139,8 +3334,11 @@
           <t>які мікрозайми подають в суд</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3171,8 +3369,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3203,8 +3404,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3235,8 +3439,11 @@
           <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>32300</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3267,8 +3474,11 @@
           <t>суд с приватбанком и как разорвать договор по кредитке</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3285,7 +3495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3294,8 +3504,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3331,10 +3542,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -3365,8 +3581,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3397,8 +3616,11 @@
           <t>чего боятся мфо украины</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>130000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3429,8 +3651,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3461,8 +3686,11 @@
           <t>как подать иск в суд на мфо</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>1810000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3493,8 +3721,11 @@
           <t>какие кредиты списывают</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3525,8 +3756,11 @@
           <t>какие кредиты списывают</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3557,8 +3791,11 @@
           <t>что такое микрокредитование и чем оно опасно</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3589,8 +3826,11 @@
           <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>32300</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3621,8 +3861,11 @@
           <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>32300</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3653,8 +3896,11 @@
           <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>32300</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3685,8 +3931,11 @@
           <t>какой максимальный процент могут начислить микрозаймы</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>32300</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3717,8 +3966,11 @@
           <t>просрочка по кредиту последствия</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>461000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3735,7 +3987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3744,8 +3996,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3781,10 +4034,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -3815,8 +4073,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3847,8 +4108,11 @@
           <t>кредитка приватбанка штраф</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>86300</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3879,8 +4143,11 @@
           <t>кредитка приватбанка штраф</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>86300</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3911,8 +4178,11 @@
           <t>кредитка приватбанка штраф</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>86300</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3943,8 +4213,11 @@
           <t>кредитка приватбанка штраф</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>86300</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -3975,8 +4248,11 @@
           <t>кредитка приватбанка штраф</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>86300</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4007,8 +4283,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4039,8 +4318,11 @@
           <t>кредитка приватбанка штраф</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>86300</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4071,8 +4353,11 @@
           <t>срок исковой давности по кредиту в приватбанке</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>1790</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4103,8 +4388,11 @@
           <t>пролонгация микрозайма</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>226000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4135,8 +4423,11 @@
           <t>оспаривание кредитного договора</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>481000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4167,8 +4458,11 @@
           <t>оспаривание кредитного договора</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>481000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4185,7 +4479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4194,8 +4488,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4231,10 +4526,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -4265,8 +4565,11 @@
           <t>переплатила кредит что делать</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>3270000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4297,8 +4600,11 @@
           <t>как вернуть часть денег за кредит</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4329,8 +4635,11 @@
           <t>нужно ли идти в банк после погашения кредита</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>3030000</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4361,8 +4670,11 @@
           <t>нужно ли писать заявление на досрочное погашение кредита</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>1920000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4393,8 +4705,11 @@
           <t>как погасить кредит если карта заблокирована</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4425,8 +4740,11 @@
           <t>можно ли погасить кредит и сразу взять новый</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>2830000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4457,8 +4775,11 @@
           <t>что делать если срок действия кредитной карты истек</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>387000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4489,8 +4810,11 @@
           <t>можно ли погасить кредит и сразу взять новый</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>2830000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4521,8 +4845,11 @@
           <t>что будет если не платить кредит за телефон</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>28900000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4553,8 +4880,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4585,8 +4915,11 @@
           <t>заявление на закрытие кредита</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>6840000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4617,8 +4950,11 @@
           <t>заявление на закрытие кредита</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>6840000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4635,7 +4971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4644,8 +4980,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4681,10 +5018,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -4715,8 +5057,11 @@
           <t>просрочка по кредиту последствия</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>461000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4747,8 +5092,11 @@
           <t>могут ли за долги посадить</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>310000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4779,8 +5127,11 @@
           <t>оспаривание кредитного договора</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>481000</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4811,8 +5162,11 @@
           <t>банк передал дело коллекторам что делать</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4843,8 +5197,11 @@
           <t>могут ли заблокировать кредитную карту приставы</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>323000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4875,8 +5232,11 @@
           <t>как уменьшить сумму платежа по кредиту</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4907,8 +5267,11 @@
           <t>можно ли не платить кредит если прошло 3 года</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>9670000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4939,8 +5302,11 @@
           <t>пришел судебный приказ о взыскании задолженности по кредиту</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>279000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -4971,8 +5337,11 @@
           <t>реструктуризация займа в микрофинансовой организации</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5003,8 +5372,11 @@
           <t>могут ли коллекторы наложить арест на имущество</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>235000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5035,8 +5407,11 @@
           <t>если муж не платит кредит что грозит жене</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>630000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5067,8 +5442,11 @@
           <t>что будет если не платить кредит под залог недвижимости</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>7180000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5085,7 +5463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5094,8 +5472,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5131,10 +5510,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -5165,8 +5549,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5197,8 +5584,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5229,8 +5619,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5261,8 +5654,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5293,8 +5689,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5325,8 +5724,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5357,8 +5759,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5389,8 +5794,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5421,8 +5829,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5453,8 +5864,11 @@
           <t>могут ли судебные приставы арестовать</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>1290000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5485,8 +5899,11 @@
           <t>как уменьшить выплаты по исполнительному листу</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>27800</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5517,8 +5934,11 @@
           <t>если есть решение суда по кредиту</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>18100000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5535,7 +5955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5544,8 +5964,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5581,10 +6002,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -5615,8 +6041,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5647,8 +6076,11 @@
           <t>влияет ли один день просрочки на кредитную историю</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>436000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5679,8 +6111,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5711,8 +6146,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5743,8 +6181,11 @@
           <t>срок исковой давности по кредиту в приватбанке</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>1790</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5775,8 +6216,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5807,8 +6251,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5839,8 +6286,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5871,8 +6321,11 @@
           <t>исправлю кредитную историю</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5903,8 +6356,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5935,8 +6391,11 @@
           <t>имеет ли право банк увеличить процент по кредиту</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>2690000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5967,8 +6426,11 @@
           <t>суд по ипотеке</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -5985,7 +6447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5994,8 +6456,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6031,10 +6494,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -6065,8 +6533,11 @@
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>1510</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6097,8 +6568,11 @@
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>1510</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6129,8 +6603,11 @@
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>1510</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6161,8 +6638,11 @@
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>1510</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6193,8 +6673,11 @@
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>1510</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6225,8 +6708,11 @@
           <t>выпустят ли за границу с долгом по кредитной карте</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>1510</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6257,8 +6743,11 @@
           <t>проверка на долги по фио</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>1570000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6289,8 +6778,11 @@
           <t>проверка на долги по фио</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>1570000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6321,8 +6813,11 @@
           <t>могут ли забрать пенсию за кредит</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>1390000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6353,8 +6848,11 @@
           <t>может ли инвалид 1 группы не платить кредит</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6385,8 +6883,11 @@
           <t>сын взял кредит и не платит что делать</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>2070000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6417,8 +6918,11 @@
           <t>что делать с кредитом если человек в тюрьме</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6435,7 +6939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6444,8 +6948,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6481,10 +6986,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -6515,8 +7025,11 @@
           <t>просрочка по кредиту последствия</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>461000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6547,8 +7060,11 @@
           <t>просрочка по кредиту последствия</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>461000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6579,8 +7095,11 @@
           <t>могут ли лишить родительских прав за неуплату кредита</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>15400</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6611,8 +7130,11 @@
           <t>могут ли кредиторы приехать домой</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6643,8 +7165,11 @@
           <t>жена набрала кредитов что делать</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>76300</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6675,8 +7200,11 @@
           <t>как скрыться от кредиторов</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>6340000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6707,8 +7235,11 @@
           <t>что делают с должниками по кредитам</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>869000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6739,8 +7270,11 @@
           <t>что делать если зарплаты не хватает на кредиты</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>1850000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6771,8 +7305,11 @@
           <t>если потерял работу как платить кредит</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>4420000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6803,8 +7340,11 @@
           <t>если муж не платит кредит что грозит жене</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>630000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6835,8 +7375,11 @@
           <t>можно ли оплачивать кредит из другой страны</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>4440000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6867,8 +7410,11 @@
           <t>может ли банк забыть про кредит</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>8180000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6885,7 +7431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6894,8 +7440,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6931,10 +7478,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -6965,8 +7517,11 @@
           <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>59800</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -6997,8 +7552,11 @@
           <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>59800</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7029,8 +7587,11 @@
           <t>как признать себя банкротом физ лицо</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>59800</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7061,8 +7622,11 @@
           <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7093,8 +7657,11 @@
           <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7125,8 +7692,11 @@
           <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7157,8 +7727,11 @@
           <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7189,8 +7762,11 @@
           <t>мой номер указали в микрозаймах</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7221,8 +7797,11 @@
           <t>заказное письмо от мфо</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>198</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7253,8 +7832,11 @@
           <t>как избавиться от звонков коллекторов по чужому кредиту</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>28400</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7285,8 +7867,11 @@
           <t>отзывы о коллекторах</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7317,8 +7902,11 @@
           <t>заказное письмо от мфо</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>198</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7335,7 +7923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7344,8 +7932,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7381,10 +7970,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -7415,8 +8009,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7447,8 +8044,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7479,8 +8079,11 @@
           <t>приватбанк списание долгов</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>4020</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7511,8 +8114,11 @@
           <t>могут ли мфо отобрать квартиру</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>272000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7543,8 +8149,11 @@
           <t>может ли мфо подать заявление в полицию</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>1520000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7575,8 +8184,11 @@
           <t>спишут ли долги по кредитам пенсионерам</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>1360000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7607,8 +8219,11 @@
           <t>какие кредиты списывают</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7639,8 +8254,11 @@
           <t>как списать долги по мфо</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>1630000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7671,8 +8289,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7703,8 +8324,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7735,8 +8359,11 @@
           <t>как оплатить только тело кредита мфо</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7767,8 +8394,11 @@
           <t>как списать долги по мфо</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>1630000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7785,7 +8415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7794,8 +8424,9 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="95" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7831,10 +8462,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Частотність кластера</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус ТЗ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Стиль</t>
         </is>
@@ -7865,8 +8501,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7897,8 +8536,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7929,8 +8571,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7961,8 +8606,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -7993,8 +8641,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8025,8 +8676,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8057,8 +8711,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8089,8 +8746,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8121,8 +8781,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8153,8 +8816,11 @@
           <t>как защитить себя от микрозаймов</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="n">
+        <v>744000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8185,8 +8851,11 @@
           <t>оспаривание кредитного договора</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="n">
+        <v>481000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
@@ -8217,8 +8886,11 @@
           <t>оспаривание кредитного договора</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n">
+        <v>481000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>

</xml_diff>

<commit_message>
Content plans: add TZ generator brief column (J) and template sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFMyDWjEn8kTss89Uu1jSY
</commit_message>
<xml_diff>
--- a/content-plans/content-plans_16-sites_nov-2026.xlsx
+++ b/content-plans/content-plans_16-sites_nov-2026.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profconsulting.com.ua" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="argument-consulting.com.ua" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spacelaw.com.ua" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шаблон ТЗ" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1035,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1047,6 +1048,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1095,6 +1097,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1130,6 +1137,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): чим небезпечний кредит під заставу квартири. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): чем опасен кредит под залог квартиры. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1165,6 +1184,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): чи можна купити квартиру якщо є борги по кредитах. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли купить квартиру если есть долги по кредитам. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1200,6 +1231,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): чи можна продати квартиру якщо є борги по кредитах. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли продать квартиру если есть долги по кредитам. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1235,6 +1278,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): як взяти відстрочку по іпотеці. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что значит заморозить займ. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1270,6 +1325,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): погана кредитна історія як взяти іпотеку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1305,6 +1372,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): як дізнатися чи знято арешт з квартири. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как проверить арест на движимое имущество. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1340,6 +1419,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): як зняти арешт з автомобіля накладений судом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как вернуть кредитную машину. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1375,6 +1466,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): чи можна продати авто яке в кредиті. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли обменять кредитную машину на другую. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1410,6 +1513,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): як перевірити чи накладено арешт на квартиру. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как проверить арест на движимое имущество. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1445,6 +1560,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): як зняти заставу з авто після погашення кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как вернуть кредитную машину. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1480,6 +1607,18 @@
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): що робити якщо на машину накладено арешт. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как вернуть кредитную машину. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1513,6 +1652,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-po-ipotechnum-kreditam.kiev.ua. Мова: українська, Україна. Автор: юрист Пономаренко Володимир Михайлович. Тематика сайту: іпотека, майнові спори, арешти майна.
+Фокусна фраза (ключ із семантики): як повернути кредитний автомобіль банку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как вернуть кредитный автомобиль банку. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: збірник «Трохи про право іпотеки» (В. Крат, Верховний Суд, 2024). Тон: спокійне авторитетне міркування судді-цивіліста; без метушні. Побудова: тезу розкладати в нумеровані абзаци (1., 2., 3.) → «Проте потрібно враховувати, що хоча …, втім …» → «Тож …». Моделювати типові ситуації («можна змоделювати випадок, коли …»). Принцип пояснювати одним реченням, інколи згадати загальний юридичний принцип. Лексика: іпотекодержатель, іпотекодавець, реєстр, відступлення права вимоги, звернення стягнення. Уникати: порад «без суду все вирішиться», жирного. Приклад: «Іпотекодержатель має право звернути стягнення на предмет іпотеки. Втім, це право не безмежне. Тож спершу перевірте, чи дотримано порядок. Можна змоделювати типовий випадок: договір є, але запису в реєстрі немає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1539,6 +1690,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1587,6 +1739,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1622,6 +1779,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як попросити в банку відстрочку за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что значит заморозить займ. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1657,6 +1826,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як отримати кредитні канікули в банку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что значит заморозить займ. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1692,6 +1873,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як оформити кредитні канікули в МФО. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что значит заморозить займ. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1727,6 +1920,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як написати лист у банк про відстрочку платежу. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что значит заморозить займ. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1762,6 +1967,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як знизити ставку за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как снизить ставку по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1797,6 +2014,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як домовитися з МФО про розстрочку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1832,6 +2061,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як домовитися з МФО про списання відсотків. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): помощь в закрытии долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1867,6 +2108,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як сплатити лише тіло кредиту МФО. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1902,6 +2155,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як закрити мікрозайм якщо немає грошей. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1937,6 +2202,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): чи можна платити мікрозайм частинами. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1972,6 +2249,18 @@
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): як краще закрити кредит достроково. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как лучше закрыть кредит досрочно. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2005,6 +2294,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту lawmsb.com.ua. Мова: українська, Україна. Автор: юрист Коваленко Володимир Сергійович. Тематика сайту: переговори з банками, реструктуризація, позасудове врегулювання боргів.
+Фокусна фраза (ключ із семантики): що означає заморозити позику. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что значит заморозить займ. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Спершу визначення двома реченнями простими словами. Далі ознаки або види, як це працює на практиці, короткий приклад і що це означає для боржника.
+Стиль автора: Джерело манери: підручник «Медіація у професійній діяльності юриста» (за ред. Крестовської, Романадзе, 2019). Тон: співпрацюючий, неконфліктний, слова про домовленість, а не про перемогу. Побудова: контраст «Традиційно … Між тим нині …» → «Однією з характерних рис є …» → інтереси й потреби сторін → кроки домовленості. Інколи колективне «ми». Банк і боржник описувати як сторони з інтересами, не як ворогів. Лексика: врегулювання, домовленість, інтереси, потреби сторін, переговори, гнучка процедура. Уникати: військової лексики («розгромити», «виграти бій»), жирного. Приклад: «Традиційно боржник бачить у банку супротивника. Між тим нині банк теж зацікавлений у домовленості. Однією з рис переговорів є гнучкість: сторони шукають інтереси, а не винних.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2031,6 +2332,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2079,6 +2381,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2114,6 +2421,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): як дізнатися чи є ти в реєстрі боржників. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как убрать себя с реестра должников. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2149,6 +2468,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): як прибрати себе з реєстру боржників. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как убрать себя с реестра должников. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2184,6 +2515,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): якщо висить борг у судових приставів. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): если висит долг у судебных приставов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2219,6 +2562,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): чи можуть заарештувати рахунки без суду. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2254,6 +2609,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): які виплати не підлягають арешту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2289,6 +2656,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): на які рахунки не можна накладати арешт. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2324,6 +2703,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): чи можна користуватися карткою якщо на ній арешт. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2359,6 +2750,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): як отримувати зарплату якщо картку арештовано. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2394,6 +2797,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): чи можна зняти арешт із зарплатної картки. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2429,6 +2844,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): як дізнатися чи арештовано рахунок. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как проверить арест на движимое имущество. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2464,6 +2891,18 @@
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): чи мають право накласти арешт на дитячу допомогу. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2497,6 +2936,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту pravovid.com.ua. Мова: українська, Україна. Автор: юрист Вишневський Сергій Олександрович. Тематика сайту: виконавче провадження, арешти рахунків і майна, реєстр боржників.
+Фокусна фраза (ключ із семантики): через скільки знімається арешт з картки після оплати. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчальний посібник «Виконавче провадження» (Ю. Білоусов, 2005). Тон: процесуальний, точний, як довідник виконавця. Побудова: «У разі …» як зачин процедури → «Відповідно до ст. … Закону …» → перелік вимог «має бути зазначено: • …; • …» → підсумок «Отже, X — це …». Кожну процедуру описувати за схемою: підстава → хто діє → строк → наслідок. Лексика: виконавчий документ, стягувач, боржник, державний виконавець, постанова. Фірмові звороти: «У разі …», «Вимоги до … встановлено …». Уникати: приблизних строків без перевірки закону, жирного. Приклад: «Постанова про арешт має містити: • дату й номер; • дані боржника; • суму стягнення. У разі невідповідності її можна оскаржити. Отже, арешт — це накладення обмеження на кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2523,6 +2974,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2571,6 +3023,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2606,6 +3063,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): як скасувати рішення суду за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как отменить решение суда по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2641,6 +3110,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): апеляція на рішення суду за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): апелляция на решение суда по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2676,6 +3157,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): що таке строк позовної давності за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): срок исковой давности по кредиту в приватбанке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Спершу визначення двома реченнями простими словами. Далі ознаки або види, як це працює на практиці, короткий приклад і що це означає для боржника.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2711,6 +3204,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): як боротися з ПриватБанком. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд с приватбанком и как разорвать договор по кредитке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2746,6 +3251,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): як дізнатися хто подав до суду за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как узнать кто подал в суд по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2781,6 +3298,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): повістка до суду за несплату кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): повестка в суд за неуплату кредита. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2816,6 +3345,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): чим загрожує суд за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): просрочка по кредиту последствия. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2851,6 +3392,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): чому банк не подає до суду за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): почему банк не подает в суд по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2886,6 +3439,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): що говорити в суді за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд по ипотеке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2921,6 +3486,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): чи можна виграти суд з банком. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд по ипотеке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2956,6 +3533,18 @@
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): як оскаржити відсотки за кредитом у суді. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2989,6 +3578,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту yuristy.in.ua. Мова: українська, Україна. Автор: юрист Хмельницький Максим Валерійович. Тематика сайту: кредитні спори, судові накази, скасування рішень, колишній юрист банків і МФО.
+Фокусна фраза (ключ із семантики): чи може суд скасувати відсотки за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: «Практикум з цивільного процесуального права України» (КНЕУ ім. Гетьмана). Тон: навчальний, діловий, через кейс-задачу. Побудова: «Ситуація» (2–3 речення з умовними даними) → «Питання: Чи може …?» → «Відповідь» із посиланням на норму та кроком дії (яку заяву подати, в який строк). Типові питання: «В якому порядку …», «Чи має право …», «Складіть заяву …». Лексика: судовий наказ, стягувач, боржник, заперечення, скасування. Уникати: вигаданих реальних клієнтів, обіцянок результату, жирного. Приклад: «Ситуація: боржник отримав судовий наказ через вісім днів. Питання: чи може він його оскаржити? Відповідь: так, протягом встановленого строку. Строк і форму заяви звіряємо за ЦПК.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3015,6 +3616,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3063,6 +3665,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -3098,6 +3705,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): банк звернувся до суду що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд по ипотеке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -3133,6 +3752,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): як поводитися в суді з банком. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд по ипотеке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3168,6 +3799,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): як оскаржити рішення суду по мікрозаймах. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3203,6 +3846,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): як виграти суд у мікрофінансової організації. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3238,6 +3893,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): як подати позов до суду на МФО. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3273,6 +3940,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): чи можна подати до суду на банк. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд по ипотеке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3308,6 +3987,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): як судитися з МФО. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3343,6 +4034,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): якщо МФО подала до суду. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): які мікрозайми подають в суд. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3378,6 +4081,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): через який час МФО подає до суду. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3413,6 +4128,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): як знизити відсотки по мікрозайму в суді. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3448,6 +4175,18 @@
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): чи нараховуються відсотки за кредитом після рішення суду. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какой максимальный процент могут начислить микрозаймы. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3481,6 +4220,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokat-kharkov.org.ua. Мова: українська, Україна. Автор: юрист Дорошенко Євгеній Сергійович. Тематика сайту: судовий захист позичальників, апеляції та касації.
+Фокусна фраза (ключ із семантики): хто судився з ПриватБанком. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд с приватбанком и как разорвать договор по кредитке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: практикум «Цивільно-процесуальне право України» (Т. Тодорошко, 2014). Тон: стислий, перевірочний, без зайвих слів. Побудова: питання-тест (чи є обов'язковою участь…?) → варіанти а) б) в) → правильна відповідь і одна норма. У статті використовувати блок «Перевірте себе» (2–3 питання) та короткі «питання — відповідь» під H2. Часто ставити прямі питання («Чи є … ?»). Лексика: апеляція, касація, строк, підстава, скарга. Уникати: довгих міркувань без питання, жирного. Приклад: «Чи можна оскаржити рішення суду після місяця? а) ні; б) так, за поважної причини; в) лише касацією. Правильно: б). Потрібне клопотання про поновлення строку.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -3495,7 +4246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3507,6 +4258,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3555,6 +4307,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -3590,6 +4347,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): що робити якщо не можеш виплатити позику. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -3625,6 +4394,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): як поводитися з МФО при простроченні. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): чего боятся мфо украины. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3660,6 +4441,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): купа боргів у МФО що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3695,6 +4488,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): що робити якщо багато позик. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как подать иск в суд на мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3730,6 +4535,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): якщо борги в кількох банках. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какие кредиты списывают. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3765,6 +4582,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): хто може допомогти з боргами. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какие кредиты списывают. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3800,6 +4629,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): що таке мікрокредитування і чим воно небезпечне. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что такое микрокредитование и чем оно опасно. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Спершу визначення двома реченнями простими словами. Далі ознаки або види, як це працює на практиці, короткий приклад і що це означає для боржника.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3835,6 +4676,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): великий борг у мікрозаймі що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какой максимальный процент могут начислить микрозаймы. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3870,6 +4723,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): скільки максимум відсотків може нарахувати МФО. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какой максимальный процент могут начислить микрозаймы. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3905,6 +4770,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): чи може пеня перевищувати суму боргу. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какой максимальный процент могут начислить микрозаймы. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3940,6 +4817,18 @@
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): чи можуть відсотки перевищувати суму позики. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какой максимальный процент могут начислить микрозаймы. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3973,6 +4862,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту profconsulting.com.ua. Мова: українська, Україна. Автор: юрист Алексєєв Олег Михайлович. Тематика сайту: кредитні спори, МФО, реструктуризація, банкрутство, боротьба з колекторами.
+Фокусна фраза (ключ із семантики): як порахувати відсоток прострочення за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): просрочка по кредиту последствия. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: посібник «Юридичні клініки на захисті прав споживачів фінансових послуг: судова практика і навички консультування» (НаУКМА, 2020). Тон: практичний аргументатор, структурований. Побудова: «Щодо недійсності …» → нумерація 1., 1.1. → норма («Відповідно до ч. 1 ст. …») → «У нашому випадку …» → «Практичні поради та способи захисту». Для кожного твердження: норма, факт, вивід. Лексика: недійсність, істотні умови, електронний підпис, доказ, позивач. Фірмові звороти: «Тож відповідно до …», «Що в нашому випадку дотримано/порушено». Уникати: загальних порад без норми, жирного. Приклад: «1. Щодо умов договору. 1.1. Електронний підпис. Одноразовим кодом підписано лише договір. Тож перевіряємо, чи охоплює підпис правила банку. У нашому випадку це означає запит журналу підписання.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -3987,7 +4888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3999,6 +4900,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4047,6 +4949,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4082,6 +4989,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): як зробити реструктуризацію кредиту в ПриватБанку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4117,6 +5036,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): борг у ПриватБанку що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): кредитка приватбанка штраф. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4152,6 +5083,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): як дізнатися чи є борг у ПриватБанку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): кредитка приватбанка штраф. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4187,6 +5130,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): як погасити кредит у ПриватБанку якщо немає грошей. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): кредитка приватбанка штраф. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4222,6 +5177,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): як нараховуються відсотки по кредитній картці ПриватБанку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): кредитка приватбанка штраф. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4257,6 +5224,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): що буде якщо не сплачувати кредитну картку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): кредитка приватбанка штраф. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4292,6 +5271,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): чи може ПриватБанк списати борг. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4327,6 +5318,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): як розрахувати обов'язковий платіж по кредитній картці ПриватБанку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): кредитка приватбанка штраф. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4362,6 +5365,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): як правильно закрити кредитку ПриватБанку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): срок исковой давности по кредиту в приватбанке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4397,6 +5412,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): що означає пролонгація кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): пролонгация микрозайма. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Спершу визначення двома реченнями простими словами. Далі ознаки або види, як це працює на практиці, короткий приклад і що це означає для боржника.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -4432,6 +5459,18 @@
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): чи можна розірвати кредитний договір з банком. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): оспаривание кредитного договора. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -4465,6 +5504,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту argument-consulting.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Тетяна Олегівна. Тематика сайту: реструктуризація кредитів, правовий аналіз договорів, кредитні картки.
+Фокусна фраза (ключ із семантики): якщо в банку немає оригіналу кредитного договору. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): оспаривание кредитного договора. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Договірне право України» (Кириченко, Кириченко, Куракін, 2024). Тон: академічно-практичний, підручниковий, багато «тобто». Побудова: поняття («Під … розуміють …») → сторони → предмет → форма → зміст/обсяг прав і обов'язків; норми цитувати з виділеним уривком «…» і номером статті; перелік умов як 1) 2) 3). Застереження «Слід зазначити, що …» та приклад у дужках «(наприклад, …)». Лексика: істотні умови, форма договору, зобов'язання, виконання, припинення. Уникати: сленгу, довгих цитат, жирного. Приклад: «Пролонгація — це продовження строку договору, тобто зміна строку, а не боргу. Слід зазначити, що змінюють договір письмово (наприклад, додатковою угодою). Сторони визначають новий графік.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -4479,7 +5530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4491,6 +5542,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4539,6 +5591,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4574,6 +5631,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): переплатила за кредитом що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): переплатила кредит что делать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4609,6 +5678,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): як повернути частину грошей за кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как вернуть часть денег за кредит. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4644,6 +5725,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): чи потрібно йти в банк після погашення кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): нужно ли идти в банк после погашения кредита. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4679,6 +5772,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): чи потрібно писати заяву на дострокове погашення кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): нужно ли писать заявление на досрочное погашение кредита. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4714,6 +5819,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): як погасити кредит якщо картку заблоковано. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как погасить кредит если карта заблокирована. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4749,6 +5866,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): чи можна погасити кредит і одразу взяти новий. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли погасить кредит и сразу взять новый. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4784,6 +5913,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): що робити якщо строк дії кредитної картки закінчився. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что делать если срок действия кредитной карты истек. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4819,6 +5960,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): чи можна погасити кредит через місяць. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли погасить кредит и сразу взять новый. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4854,6 +6007,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): що буде якщо не платити кредит за телефон. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что будет если не платить кредит за телефон. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4889,6 +6054,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): чи може банк списати борг за кредитом із зарплатної картки. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -4924,6 +6101,18 @@
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): які документи потрібні для закриття кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): заявление на закрытие кредита. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -4957,6 +6146,162 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту spacelaw.com.ua. Мова: українська, Україна. Автор: юрист Олійник Євгенія Леонідівна. Тематика сайту: банківське право, кредитні спори, закриття та погашення кредитів.
+Фокусна фраза (ключ із семантики): як взяти довідку про закриття кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): заявление на закрытие кредита. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (Х. Бехруз, К. Мануїлова; за ред. О. Дмитрик, НЮУ, 2022). Тон: нормативний, послідовний, без розмовності. Побудова: «Відповідно до …» → коротка цитата норми у лапках → «При цьому …» → «Отже, підставами/умовами є …»; «У разі …» як початок правил; «Так само …» для аналогій. Складні поняття розкладати на підстави й обмеження. Лексика: позичальник, заборгованість, погашення, списання, кредитні кошти. Уникати: розмовних слів, оцінок, жирного. Приклад: «Відповідно до закону, списання коштів потребує підстави. При цьому підставою може бути договір або рішення суду. Отже, спершу перевірте, на якій підставі списали кошти.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Частина</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Текст</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Фокусна фраза</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Фокусна фраза (ключ із семантики): </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Кластер</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): </t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Читач і структура</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Структура: чи</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Структура: як</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Структура: що таке</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Спершу визначення двома реченнями простими словами. Далі ознаки або види, як це працює на практиці, короткий приклад і що це означає для боржника.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Структура: інше</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Стиль</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Стиль автора: </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Кінець</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -4971,7 +6316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4983,6 +6328,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5031,6 +6377,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -5066,6 +6417,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): що буде за прострочення кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): просрочка по кредиту последствия. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -5101,6 +6464,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): чи можуть за борги посадити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли за долги посадить. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -5136,6 +6511,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): як оскаржити кредитний договір з банком. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): оспаривание кредитного договора. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -5171,6 +6558,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): банк передав справу колекторам що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): банк передал дело коллекторам что делать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -5206,6 +6605,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): чи можуть заблокувати кредитну картку пристави. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли заблокировать кредитную карту приставы. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -5241,6 +6652,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): як зменшити суму платежу за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить сумму платежа по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -5276,6 +6699,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): чи можна не платити кредит якщо минуло 3 роки. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли не платить кредит если прошло 3 года. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -5311,6 +6746,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): прийшов судовий наказ про стягнення заборгованості за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): пришел судебный приказ о взыскании задолженности по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -5346,6 +6793,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): як реструктуризувати мікрозайми. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): реструктуризация займа в микрофинансовой организации. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -5381,6 +6840,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): чи можуть колектори накласти арешт на майно. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли коллекторы наложить арест на имущество. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -5416,6 +6887,18 @@
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): якщо чоловік не платить кредит що загрожує дружині. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): если муж не платит кредит что грозит жене. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -5449,6 +6932,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту legaladdress.com.ua. Мова: українська, Україна. Автор: юрист Бойчук Артем Валерійович. Тематика сайту: юрист по кредитах: аналіз договору, переговори з банком, колектори, суд, іпотека.
+Фокусна фраза (ключ із семантики): що буде якщо не платити кредит під заставу нерухомості. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что будет если не платить кредит под залог недвижимости. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник цивільного права (Борисова та ін., за ТЗ). Тон: спокійний, академічний, від першої особи юриста. Побудова: визначення «X — це …» → класифікація («за підставою … поділяються на …») → застереження «хоча …, однак …». Під кожним H2 пряма відповідь на 40–60 слів. Лексика: правочин, істотні умови, кредитодавець, позичальник; без розмовних слів. Фірмові звороти: «Розрізняють три види …», «Слід відрізняти … від …». Уникати: категоричних обіцянок, жирного, канцеляризмів. Приклад: «Кредитні канікули — це відстрочка платежів за домовленістю з банком. Борг при цьому не списується. Розрізняють три види таких канікул.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -5463,7 +6958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5475,6 +6970,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5523,6 +7019,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -5558,6 +7059,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): що буде якщо не платити за виконавчим листом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -5593,6 +7106,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): чи можна домовитися з приставами. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -5628,6 +7153,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): що робити якщо прийшов виконавчий лист за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -5663,6 +7200,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): як зменшити виплати за виконавчим листом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -5698,6 +7247,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): як скасувати виконавче провадження за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -5733,6 +7294,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): як припинити виконавче провадження якщо борг погашено. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -5768,6 +7341,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): чи можна скасувати виконавчий лист. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -5803,6 +7388,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): як закрити заборгованість у приставів. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -5838,6 +7435,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): як не платити борг за рішенням суду. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -5873,6 +7482,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): чи можуть пристави знімати всі гроші із зарплатної картки. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли судебные приставы арестовать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -5908,6 +7529,18 @@
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): що робити з виконавчим листом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как уменьшить выплаты по исполнительному листу. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -5941,6 +7574,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту rada-advokat.uz.ua. Мова: українська, Україна. Автор: юрист Кравченко Максим Віталійович. Тематика сайту: кредитні спори, виконавче провадження, примусове стягнення, МФО і колектори.
+Фокусна фраза (ключ із семантики): якщо є рішення суду за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): если есть решение суда по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: навчально-методичний посібник «Банківське право» (Лаврик, Терела, за ТЗ). Тон: офіційно-нормативний, нейтральний. Побудова: «Відповідно до …» → що вимагає норма → наслідок для боржника; чітка структура теми, переліки через «;» («1) …; 2) …;»). Посилання на закон у дужках. Лексика: кредитодавець, споживач, примусове стягнення, виконавче провадження. Фірмові звороти: «Відповідно до закону …», «У разі … боржник має право …». Уникати: емоцій, розмовних порад, обіцянок результату. Приклад: «Відповідно до закону, колектор називає себе й підставу звернення. Вимагайте письмово: 1) договір про відступлення права; 2) розрахунок боргу; 3) підтвердження повноважень.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -5955,7 +7600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5967,6 +7612,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6015,6 +7661,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -6050,6 +7701,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): як виправити кредитну історію якщо були прострочення. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -6085,6 +7748,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): чи впливає один день прострочення на кредитну історію. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): влияет ли один день просрочки на кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -6120,6 +7795,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): чи впливає судова заборгованість на кредитну історію. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -6155,6 +7842,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): скільки зберігається кредитна історія в Україні. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -6190,6 +7889,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): через скільки згорає кредитна історія. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): срок исковой давности по кредиту в приватбанке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -6225,6 +7936,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): якщо є прострочення за кредитом чи дадуть кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -6260,6 +7983,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): чому мені не дають кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -6295,6 +8030,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): якщо не платити кредит через скільки він анулюється. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -6330,6 +8077,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): як дізнатися чи є в мене кредити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): исправлю кредитную историю. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -6365,6 +8124,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): чи може банк вимагати повернути весь кредит одразу. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -6400,6 +8171,18 @@
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): чи має право банк збільшити відсоток за кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): имеет ли право банк увеличить процент по кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -6433,6 +8216,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту ukrjurist.com.ua. Мова: українська, Україна. Автор: юрист Гончарук Вікторія Анатолівна. Тематика сайту: юрист по кредитах: кредитна історія, дії банку, права позичальника.
+Фокусна фраза (ключ із семантики): як оскаржити комісію банку. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): суд по ипотеке. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: огляд практики Верховного Суду (за ТЗ). Тон: стримано-аналітичний, довіра через номери справ і дати. Побудова блоку: «Позиція суду» → «Що це означає для вас» → «Детальніше: справа № …, дата …». Номери справ і дати брати лише після прочитання рішення в ЄДРСР. Лексика: касаційний суд, правова позиція, відступ від позиції, доказування. Фірмові звороти: «Суд зазначив, що …», «Це означає, що …». Уникати: узагальнень без справи, жирного, «адвокат» (на сайті «юрист по кредитам»). Приклад: «Позиція суду: банк має довести правомірність блокування. Що це означає: клієнт вимагає причину письмово. Детальніше: справа № [ПЕРЕВІРИТИ], [дата].» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -6447,7 +8242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6459,6 +8254,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6507,6 +8303,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -6542,6 +8343,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): чи можна виїхати з України якщо є кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): выпустят ли за границу с долгом по кредитной карте. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -6577,6 +8390,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): чи випустять за кордон з боргом по кредитній картці. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): выпустят ли за границу с долгом по кредитной карте. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -6612,6 +8437,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): з якою сумою заборгованості не випускають за кордон. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): выпустят ли за границу с долгом по кредитной карте. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -6647,6 +8484,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): як перевірити чи є борги для виїзду за кордон. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): выпустят ли за границу с долгом по кредитной карте. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -6682,6 +8531,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): чи можуть колектори заборонити виїзд за кордон. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): выпустят ли за границу с долгом по кредитной карте. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -6717,6 +8578,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): чи випустять за кордон з іпотекою. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): выпустят ли за границу с долгом по кредитной карте. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -6752,6 +8625,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): як дізнатися борги за прізвищем. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): проверка на долги по фио. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -6787,6 +8672,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): як дізнатися всі свої борги по кредитах. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): проверка на долги по фио. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -6822,6 +8719,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): чи можуть забрати пенсію за кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли забрать пенсию за кредит. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -6857,6 +8766,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): чи може інвалід 1 групи не платити кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): может ли инвалид 1 группы не платить кредит. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -6892,6 +8813,18 @@
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): син узяв кредит і не платить що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): сын взял кредит и не платит что делать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -6925,6 +8858,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту uchet.com.ua. Мова: українська, Україна. Автор: юрист Борисов Максим Юрійович. Тематика сайту: юрист по кредитах: виїзд за кордон з боргами, перевірка боргів, сімейні ситуації.
+Фокусна фраза (ключ із семантики): що робити з кредитом якщо людина у в'язниці. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что делать с кредитом если человек в тюрьме. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник сімейного права (Апопій, за ТЗ). Тон: теплий, але чіткий, розмовна прямота без панібратства. Побудова: «по-перше / по-друге / по-третє» → норма → виняток («Проте …») → приклад «Так, …». Короткі приклади з життя без вигаданих клієнтів. Лексика: простіша, ніж у законі: «арешт», «картка», «виплата». Фірмові звороти: «Загальне правило таке …», «Проте є виняток …», «Так, …». Уникати: довгих цитат норм, жирного, накопичення термінів. Приклад: «Арешт не дорівнює списанню. По-перше, виконавець накладає арешт постановою. По-друге, гроші залишаються на рахунку. Проте є виняток: на деякі виплати арешт не поширюється.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -6939,7 +8884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6951,6 +8896,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6999,6 +8945,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -7034,6 +8985,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): чи можуть звільнити за борги по кредитах. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): просрочка по кредиту последствия. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -7069,6 +9032,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): чи можуть забрати права за несплату кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): просрочка по кредиту последствия. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -7104,6 +9079,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): чи можуть позбавити батьківських прав за несплату кредиту. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли лишить родительских прав за неуплату кредита. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -7139,6 +9126,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): чи можуть кредитори приїхати додому. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли кредиторы приехать домой. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -7174,6 +9173,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): дружина набрала кредитів що робити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): жена набрала кредитов что делать. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -7209,6 +9220,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): як сховатися від кредиторів. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как скрыться от кредиторов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -7244,6 +9267,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): що роблять з боржниками по кредитах. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что делают с должниками по кредитам. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -7279,6 +9314,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): що робити якщо зарплати не вистачає на кредити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): что делать если зарплаты не хватает на кредиты. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -7314,6 +9361,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): якщо втратив роботу як платити кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): если потерял работу как платить кредит. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -7349,6 +9408,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): якщо не виплачувати кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): если муж не платит кредит что грозит жене. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -7384,6 +9455,18 @@
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): чи можна сплачувати кредит з-за кордону. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): можно ли оплачивать кредит из другой страны. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -7417,6 +9500,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту urists.com.ua. Мова: українська, Україна. Автор: юрист Яковенко Дмитро. Тематика сайту: юрист по кредитах: права боржника, роботодавець, родичі, колектори вдома.
+Фокусна фраза (ключ із семантики): чи може банк забути про кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): может ли банк забыть про кредит. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник кримінального процесу та правничої допомоги (Тертишник, за ТЗ). Тон: ділово-оцінний, впевнений. Побудова: широкий контекст → нумерована група умов 1) 2) 3) → висновок; оцінні формулювання «незважаючи на … містять …». Умови та підстави завжди нумерувати. Лексика: ухилення від виконання, обмеження права, підстава, умова. Фірмові звороти: «Обмеження застосовують за трьох умов: …», «Отже, ключовою є умова …». Уникати: розмитих «може бути», жирного. Приклад: «Суд обмежує виїзд лише за умов: 1) боржник ухиляється від виконання; 2) виконавець звертається до суду; 3) суд постановляє ухвалу. Отже, сам кредит заборони не створює.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -7431,7 +9526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7443,6 +9538,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7491,6 +9587,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -7526,6 +9627,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): як визнати себе банкрутом фізична особа. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как признать себя банкротом физ лицо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -7561,6 +9674,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): що якщо оголосити себе банкрутом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как признать себя банкротом физ лицо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -7596,6 +9721,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): що потрібно щоб оголосити себе банкрутом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как признать себя банкротом физ лицо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -7631,6 +9768,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): як колектори знаходять родичів. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): мой номер указали в микрозаймах. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -7666,6 +9815,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): як колектори дізнаються адресу. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): мой номер указали в микрозаймах. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -7701,6 +9862,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): що буде якщо не брати слухавку від колекторів. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): мой номер указали в микрозаймах. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -7736,6 +9909,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): що можуть зробити колектори родичам боржника. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): мой номер указали в микрозаймах. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -7771,6 +9956,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): як зупинити дзвінки колекторів. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): мой номер указали в микрозаймах. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -7806,6 +10003,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): чи можуть колектори продати борг іншим колекторам. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): заказное письмо от мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -7841,6 +10050,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): як позбутися дзвінків колекторів за чужим кредитом. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как избавиться от звонков коллекторов по чужому кредиту. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -7876,6 +10097,18 @@
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): хто такий антиколектор. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): отзывы о коллекторах. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -7909,6 +10142,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту advokato.in.ua. Мова: українська, Україна. Автор: юрист Коваленко Наталія Олександрівна. Тематика сайту: колектори та банкрутство фізосіб.
+Фокусна фраза (ключ із семантики): як розмовляти з колекторами якщо немає грошей. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): заказное письмо от мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Аналіз судової практики інституту неплатоспроможності фізичних осіб» (Г. Григорян, проєкт PRAVO-Justice, ЄС, 2021). Тон: аналітичний, експертний, без пафосу. Побудова: проблема → як по-різному вирішують суди («Аналогічний висновок робить суд у справі № …») → «Отже, є підстави вважати, що …» → «Рекомендації». Умовний приклад із сумою цифрами й словами («10 000 (десять тисяч) гривень»), позначений як ілюстрація. Риторичне питання на початку: «Чи є …?». Лексика: неплатоспроможність, план реструктуризації, кредитор, зборами кредиторів. Уникати: оцінок без справи, жирного. Приклад: «Чи може кредитор змінити голосування, відмовившись від застави? Суди відповідають по-різному. Отже, є підстави вважати, що важливий розмір вимог. Рекомендація: перевірте реєстр вимог.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -7923,7 +10168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7935,6 +10180,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7983,6 +10229,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -8018,6 +10269,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): як списати борги по кредитній картці. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -8053,6 +10316,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): як законно списати кредити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -8088,6 +10363,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): коли спишуть кредити. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): приватбанк списание долгов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -8123,6 +10410,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): чи можуть МФО забрати квартиру. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): могут ли мфо отобрать квартиру. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -8158,6 +10457,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): чи може МФО подати заяву в поліцію. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): может ли мфо подать заявление в полицию. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -8193,6 +10504,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): чи спишуть борги по кредитах пенсіонерам. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): спишут ли долги по кредитам пенсионерам. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -8228,6 +10551,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): які кредити списують. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): какие кредиты списывают. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -8263,6 +10598,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): чи можуть МФО пробачити борг. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как списать долги по мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -8298,6 +10645,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): як позбутися кредитних боргів законно. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -8333,6 +10692,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): як списати відсотки по мікрозайму. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -8368,6 +10739,18 @@
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): як дізнатися чи списали мені кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как оплатить только тело кредита мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -8401,6 +10784,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту bankruptcyukraine.com. Мова: українська, Україна. Автор: юрист Бондар Олег Олексійович. Тематика сайту: списання боргів, приватні кредитори, МФО.
+Фокусна фраза (ключ із семантики): куди звернутися щоб списали кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как списать долги по мфо. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: підручник «Фінансове право» (за ред. Кучерявенка, Дмитрик, НЮУ, 2019). Тон: доктринальний, але зрозумілий; авторське «ми/додамо». Побудова: теза → пояснення методу/принципу → «До цього додамо, що …» → «До того ж можна стверджувати і про зворотний вплив …» → «Таким чином …». Роль приватного кредитора й держави пояснювати через принцип, а потім практику. Лексика: правовідносини, суб'єкт, імперативний, диспозитивність (давати простішим словом). Фірмові звороти: «Слід наголосити, що …», «Отже, …». Уникати: теоретичних відступів без практичного висновку, жирного. Приклад: «Слід наголосити: списання боргу — це правова процедура, а не втеча від кредитора. До цього додамо, що закон ставить умови. Отже, спершу з'ясуємо, чи боржник їм відповідає.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>
@@ -8415,7 +10810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8427,6 +10822,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="95" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8475,6 +10871,11 @@
           <t>Стиль</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Опис для генератора ТЗ (вставити в поле «Опишіть особливості контенту»)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -8510,6 +10911,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): як дізнатися чи взято на мене мікрозайм. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -8545,6 +10958,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): що робити якщо на тебе оформили мікрозайм. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -8580,6 +11005,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): чи можуть оформити кредит без мого відома. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -8615,6 +11052,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): як захиститися від кредитних шахраїв. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -8650,6 +11099,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): що робити якщо шахраї змусили взяти кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -8685,6 +11146,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): як довести що ти не брав кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -8720,6 +11193,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): як оскаржити кредит який не брав. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -8755,6 +11240,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): дзвонять кажуть що на вас оформлено кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -8790,6 +11287,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): чи безпечно брати позику через інтернет. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Відповідь на запит дати одразу в першому абзаці: так, ні або залежить від обставин, і одним реченням чому. Далі розкрити, за яких умов так, за яких ні, які є винятки і що робити читачеві.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -8825,6 +11334,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): куди звертатися якщо на мене оформили кредит. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): как защитить себя от микрозаймов. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -8860,6 +11381,18 @@
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): як визнати договір з МФО недійсним. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): оспаривание кредитного договора. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Короткий підсумок способу дати одразу в першому абзаці. Далі покрокова інструкція нумерованим списком: що підготувати, куди звертатися, у які строки, типові помилки.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -8893,6 +11426,18 @@
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тип: інформаційна стаття для блогу сайту jurist-online.info. Мова: українська, Україна. Автор: юрист Мельник Марія Миколаївна. Тематика сайту: захист прав споживачів кредитних послуг, МФО, шахрайські кредити.
+Фокусна фраза (ключ із семантики): що робити якщо втратив кредитний договір. Вжити її в заголовку H1, у першому абзаці й в одному підзаголовку, природно, без переспаму.
+Суміжний кластер семантики (як у семантиці, російською): оспаривание кредитного договора. Враховувати як контекст, окремою темою не робити.
+Читач: людина з проблемою за кредитом чи боргом, шукає чітку відповідь без юридичного жаргону.
+Структура: Коротку відповідь і головну дію дати одразу в першому абзаці. Далі: що відбувається за законом, які права має читач, покрокові дії, чого не робити, коли потрібен юрист.
+Стиль автора: Джерело манери: «Порадник клініциста: правила надання правової допомоги споживачам фінансових послуг» (ЧНУ ім. Федьковича). Тон: практичний, допомагаючий, звернення на «Ви». Побудова: «Алгоритм дій» → нумеровані кроки → питання-тест до читача («Чи підписували ви договір?») → норма короткою цитатою («Відповідно до … закону …») → зразок документа. Пояснення починати з ситуації споживача, не з норми. Лексика: споживач, фінансова послуга, кредитодавець, претензія. Фірмові звороти: «Крок 1. З'ясуйте …», «Тест на …», «Перевірте себе: …». Уникати: теорії без дії, жирного. Приклад: «Крок 1. З'ясуйте, чи брали ви цей кредит. Запитайте себе: чи підписували договір? Чи приходив код у СМС? Крок 2. Надішліть запит до бюро кредитних історій.» Правила головреда для всіх: речення 5–14 слів (проза до 20), без жирного, прямий висновок на початку розділу. З книжки беремо лише манеру, не теми й не цитати. Приклади лише ілюструють манеру: факти й норми звіряти.
+Обов'язково: блок питань і відповідей на 3-5 запитань; на норми закону посилатися лише там, де впевнені, інакше без номера статті; зазначити, що остаточне рішення залежить від документів у конкретній справі; наприкінці короткий заклик звернутися до юриста за консультацією. Обсяг орієнтовно 5000-7000 знаків із пробілами.
+Уникати: обіцянок виграти справу чи гарантій результату, вигаданих цифр, судових справ і статистики без джерела, цін на послуги.</t>
         </is>
       </c>
     </row>

</xml_diff>